<commit_message>
add sheet layout into template DD
</commit_message>
<xml_diff>
--- a/design-detail/DD_Staff_v1.0.xlsx
+++ b/design-detail/DD_Staff_v1.0.xlsx
@@ -8,47 +8,49 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Course-management\Source\course-management\design-detail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD1B36A-68EA-4B7E-8CB6-D354639FEC0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA9ABA2-1DEB-4ADC-88FF-76C482C73E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="780" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="His" sheetId="32" r:id="rId1"/>
-    <sheet name="Overview" sheetId="28" r:id="rId2"/>
-    <sheet name="SQL" sheetId="35" r:id="rId3"/>
-    <sheet name="ClassDiagram" sheetId="42" r:id="rId4"/>
-    <sheet name="SequenceDiagram" sheetId="43" r:id="rId5"/>
-    <sheet name="APIs" sheetId="36" r:id="rId6"/>
-    <sheet name="Sheet3" sheetId="34" state="hidden" r:id="rId7"/>
+    <sheet name="Layout" sheetId="45" r:id="rId2"/>
+    <sheet name="Overview" sheetId="28" r:id="rId3"/>
+    <sheet name="SQL" sheetId="35" r:id="rId4"/>
+    <sheet name="ClassDiagram" sheetId="42" r:id="rId5"/>
+    <sheet name="SequenceDiagram" sheetId="43" r:id="rId6"/>
+    <sheet name="APIs" sheetId="36" r:id="rId7"/>
+    <sheet name="Sheet3" sheetId="34" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
+    <definedName name="_Key1" localSheetId="6" hidden="1">#REF!</definedName>
+    <definedName name="_Key1" localSheetId="4" hidden="1">#REF!</definedName>
+    <definedName name="_Key1" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Key1" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Key1" localSheetId="3" hidden="1">#REF!</definedName>
-    <definedName name="_Key1" localSheetId="0" hidden="1">#REF!</definedName>
-    <definedName name="_Key1" localSheetId="4" hidden="1">#REF!</definedName>
-    <definedName name="_Key1" localSheetId="2" hidden="1">#REF!</definedName>
     <definedName name="_Key1" hidden="1">#REF!</definedName>
     <definedName name="_Order1" hidden="1">255</definedName>
+    <definedName name="_Regression_X" localSheetId="6" hidden="1">#REF!</definedName>
+    <definedName name="_Regression_X" localSheetId="4" hidden="1">#REF!</definedName>
     <definedName name="_Regression_X" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Regression_X" localSheetId="3" hidden="1">#REF!</definedName>
-    <definedName name="_Regression_X" localSheetId="4" hidden="1">#REF!</definedName>
-    <definedName name="_Regression_X" localSheetId="2" hidden="1">#REF!</definedName>
     <definedName name="_Regression_X" hidden="1">#REF!</definedName>
+    <definedName name="_Sort" localSheetId="6" hidden="1">#REF!</definedName>
+    <definedName name="_Sort" localSheetId="4" hidden="1">#REF!</definedName>
     <definedName name="_Sort" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Sort" localSheetId="3" hidden="1">#REF!</definedName>
-    <definedName name="_Sort" localSheetId="4" hidden="1">#REF!</definedName>
-    <definedName name="_Sort" localSheetId="2" hidden="1">#REF!</definedName>
     <definedName name="_Sort" hidden="1">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">APIs!$A$1:$BT$66</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">ClassDiagram!$A$1:$BG$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">APIs!$A$1:$BT$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">ClassDiagram!$A$1:$BG$35</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">His!$A$1:$E$23</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">SequenceDiagram!$A$1:$BG$30</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">SQL!$A$1:$BG$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Layout!$A$1:$BL$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">SequenceDiagram!$A$1:$BG$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">SQL!$A$1:$BG$26</definedName>
+    <definedName name="関連表" localSheetId="6" hidden="1">#REF!</definedName>
+    <definedName name="関連表" localSheetId="4" hidden="1">#REF!</definedName>
+    <definedName name="関連表" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="関連表" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="関連表" localSheetId="3" hidden="1">#REF!</definedName>
-    <definedName name="関連表" localSheetId="0" hidden="1">#REF!</definedName>
-    <definedName name="関連表" localSheetId="4" hidden="1">#REF!</definedName>
-    <definedName name="関連表" localSheetId="2" hidden="1">#REF!</definedName>
     <definedName name="関連表" hidden="1">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -67,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="111">
   <si>
     <t>Label</t>
   </si>
@@ -401,6 +403,9 @@
   </si>
   <si>
     <t>Update</t>
+  </si>
+  <si>
+    <t>figma</t>
   </si>
 </sst>
 </file>
@@ -2093,6 +2098,147 @@
     <xf numFmtId="0" fontId="49" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="38" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="29" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="28" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="37" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="37" borderId="4" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="4" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="21" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="37" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="37" borderId="4" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="4" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="21" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="24" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="22" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="23" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="18" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="15" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="19" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="37" borderId="21" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="20" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="20" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="4" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="21" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="24" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="22" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="23" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="18" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="15" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="19" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="22" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="23" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="15" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="19" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="37" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="37" borderId="4" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="47" fillId="37" borderId="21" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="38" borderId="26" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="38" borderId="4" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="38" borderId="25" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="41" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="43" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="40" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="24" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="18" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="22" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="18" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="15" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="49" fontId="47" fillId="0" borderId="39" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2105,145 +2251,13 @@
     <xf numFmtId="49" fontId="47" fillId="0" borderId="42" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="24" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="22" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="4" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="23" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="18" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="15" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="19" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="24" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="22" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="23" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="18" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="15" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="19" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="24" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="22" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="18" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="15" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="38" borderId="26" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="38" borderId="4" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="38" borderId="25" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="38" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="29" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="28" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="41" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="43" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="40" xfId="76" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="37" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="37" borderId="4" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="37" borderId="4" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="37" borderId="21" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="37" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="37" borderId="4" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="37" borderId="4" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="37" borderId="21" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="37" borderId="21" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="37" borderId="20" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="37" borderId="20" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="37" borderId="4" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="37" borderId="21" xfId="130" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="22" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="23" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="18" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="15" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="19" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="37" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="37" borderId="4" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="37" borderId="21" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="47" fillId="0" borderId="21" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="47" fillId="0" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2264,14 +2278,38 @@
     <xf numFmtId="0" fontId="47" fillId="0" borderId="20" xfId="130" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="20" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="4" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="47" fillId="0" borderId="21" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="40" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="40" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="40" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="40" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="40" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="40" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="37" borderId="16" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="37" borderId="0" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="0" borderId="8" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2290,39 +2328,6 @@
     </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="21" xfId="133" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="40" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="40" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="40" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="40" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="40" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="40" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="37" borderId="16" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="37" borderId="0" xfId="130" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="8" xfId="130" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="144">
@@ -2493,6 +2498,55 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>30939</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>7950</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C0CD704-5B59-716D-15CC-16A198511146}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="998220" y="1531620"/>
+          <a:ext cx="5296359" cy="3810330"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>45720</xdr:colOff>
       <xdr:row>12</xdr:row>
@@ -2538,7 +2592,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2587,7 +2641,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -3182,11 +3236,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{222134E3-A126-43B4-9320-68F74CBADA6F}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BM25"/>
+  <dimension ref="A1:BM9"/>
   <sheetFormatPr defaultColWidth="2.33203125" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="3.109375" style="2" customWidth="1"/>
@@ -3203,248 +3257,248 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:65" s="5" customFormat="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="134" t="s">
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="139" t="s">
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="119" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="136"/>
-      <c r="M1" s="136"/>
-      <c r="N1" s="136"/>
-      <c r="O1" s="137"/>
-      <c r="P1" s="140" t="s">
+      <c r="L1" s="109"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="120" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="141"/>
-      <c r="R1" s="141"/>
-      <c r="S1" s="141"/>
-      <c r="T1" s="142"/>
-      <c r="U1" s="140" t="s">
+      <c r="Q1" s="121"/>
+      <c r="R1" s="121"/>
+      <c r="S1" s="121"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="120" t="s">
         <v>15</v>
       </c>
-      <c r="V1" s="141"/>
-      <c r="W1" s="141"/>
-      <c r="X1" s="141"/>
-      <c r="Y1" s="141"/>
-      <c r="Z1" s="141"/>
-      <c r="AA1" s="141"/>
-      <c r="AB1" s="141"/>
-      <c r="AC1" s="141"/>
-      <c r="AD1" s="141"/>
-      <c r="AE1" s="141"/>
-      <c r="AF1" s="141"/>
-      <c r="AG1" s="141"/>
-      <c r="AH1" s="142"/>
-      <c r="AI1" s="148" t="s">
+      <c r="V1" s="121"/>
+      <c r="W1" s="121"/>
+      <c r="X1" s="121"/>
+      <c r="Y1" s="121"/>
+      <c r="Z1" s="121"/>
+      <c r="AA1" s="121"/>
+      <c r="AB1" s="121"/>
+      <c r="AC1" s="121"/>
+      <c r="AD1" s="121"/>
+      <c r="AE1" s="121"/>
+      <c r="AF1" s="121"/>
+      <c r="AG1" s="121"/>
+      <c r="AH1" s="122"/>
+      <c r="AI1" s="133" t="s">
         <v>16</v>
       </c>
-      <c r="AJ1" s="149"/>
-      <c r="AK1" s="149"/>
-      <c r="AL1" s="149"/>
-      <c r="AM1" s="150"/>
-      <c r="AN1" s="148" t="s">
+      <c r="AJ1" s="134"/>
+      <c r="AK1" s="134"/>
+      <c r="AL1" s="134"/>
+      <c r="AM1" s="135"/>
+      <c r="AN1" s="133" t="s">
         <v>17</v>
       </c>
-      <c r="AO1" s="149"/>
-      <c r="AP1" s="149"/>
-      <c r="AQ1" s="149"/>
-      <c r="AR1" s="150"/>
-      <c r="AS1" s="148" t="s">
+      <c r="AO1" s="134"/>
+      <c r="AP1" s="134"/>
+      <c r="AQ1" s="134"/>
+      <c r="AR1" s="135"/>
+      <c r="AS1" s="133" t="s">
         <v>18</v>
       </c>
-      <c r="AT1" s="149"/>
-      <c r="AU1" s="149"/>
-      <c r="AV1" s="149"/>
-      <c r="AW1" s="150"/>
-      <c r="AX1" s="134" t="s">
+      <c r="AT1" s="134"/>
+      <c r="AU1" s="134"/>
+      <c r="AV1" s="134"/>
+      <c r="AW1" s="135"/>
+      <c r="AX1" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="AY1" s="136"/>
-      <c r="AZ1" s="136"/>
-      <c r="BA1" s="136"/>
-      <c r="BB1" s="137"/>
-      <c r="BC1" s="134" t="s">
+      <c r="AY1" s="109"/>
+      <c r="AZ1" s="109"/>
+      <c r="BA1" s="109"/>
+      <c r="BB1" s="110"/>
+      <c r="BC1" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="BD1" s="135"/>
-      <c r="BE1" s="135"/>
-      <c r="BF1" s="136"/>
-      <c r="BG1" s="137"/>
-      <c r="BH1" s="130" t="s">
+      <c r="BD1" s="108"/>
+      <c r="BE1" s="108"/>
+      <c r="BF1" s="109"/>
+      <c r="BG1" s="110"/>
+      <c r="BH1" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="BI1" s="131"/>
-      <c r="BJ1" s="132"/>
-      <c r="BK1" s="132"/>
-      <c r="BL1" s="133"/>
+      <c r="BI1" s="104"/>
+      <c r="BJ1" s="105"/>
+      <c r="BK1" s="105"/>
+      <c r="BL1" s="106"/>
       <c r="BM1" s="2"/>
     </row>
     <row r="2" spans="1:65" s="5" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A2" s="116" t="s">
+      <c r="A2" s="123" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="143"/>
-      <c r="C2" s="143"/>
-      <c r="D2" s="143"/>
-      <c r="E2" s="144"/>
-      <c r="F2" s="116" t="s">
+      <c r="B2" s="124"/>
+      <c r="C2" s="124"/>
+      <c r="D2" s="124"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="123" t="s">
         <v>58</v>
       </c>
-      <c r="G2" s="143"/>
-      <c r="H2" s="143"/>
-      <c r="I2" s="143"/>
-      <c r="J2" s="144"/>
-      <c r="K2" s="105" t="s">
+      <c r="G2" s="124"/>
+      <c r="H2" s="124"/>
+      <c r="I2" s="124"/>
+      <c r="J2" s="125"/>
+      <c r="K2" s="129" t="s">
         <v>54</v>
       </c>
-      <c r="L2" s="105"/>
-      <c r="M2" s="105"/>
-      <c r="N2" s="105"/>
-      <c r="O2" s="106"/>
-      <c r="P2" s="104" t="s">
+      <c r="L2" s="129"/>
+      <c r="M2" s="129"/>
+      <c r="N2" s="129"/>
+      <c r="O2" s="130"/>
+      <c r="P2" s="142" t="s">
         <v>55</v>
       </c>
-      <c r="Q2" s="105"/>
-      <c r="R2" s="105"/>
-      <c r="S2" s="105"/>
-      <c r="T2" s="106"/>
-      <c r="U2" s="104" t="s">
+      <c r="Q2" s="129"/>
+      <c r="R2" s="129"/>
+      <c r="S2" s="129"/>
+      <c r="T2" s="130"/>
+      <c r="U2" s="142" t="s">
         <v>52</v>
       </c>
-      <c r="V2" s="105"/>
-      <c r="W2" s="105"/>
-      <c r="X2" s="105"/>
-      <c r="Y2" s="105"/>
-      <c r="Z2" s="105"/>
-      <c r="AA2" s="105"/>
-      <c r="AB2" s="105"/>
-      <c r="AC2" s="105"/>
-      <c r="AD2" s="105"/>
-      <c r="AE2" s="105"/>
-      <c r="AF2" s="105"/>
-      <c r="AG2" s="105"/>
-      <c r="AH2" s="106"/>
-      <c r="AI2" s="110">
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
+      <c r="Z2" s="129"/>
+      <c r="AA2" s="129"/>
+      <c r="AB2" s="129"/>
+      <c r="AC2" s="129"/>
+      <c r="AD2" s="129"/>
+      <c r="AE2" s="129"/>
+      <c r="AF2" s="129"/>
+      <c r="AG2" s="129"/>
+      <c r="AH2" s="130"/>
+      <c r="AI2" s="111">
         <v>45701</v>
       </c>
-      <c r="AJ2" s="111"/>
-      <c r="AK2" s="111"/>
-      <c r="AL2" s="111"/>
-      <c r="AM2" s="112"/>
-      <c r="AN2" s="116" t="s">
+      <c r="AJ2" s="112"/>
+      <c r="AK2" s="112"/>
+      <c r="AL2" s="112"/>
+      <c r="AM2" s="113"/>
+      <c r="AN2" s="123" t="s">
         <v>56</v>
       </c>
-      <c r="AO2" s="117"/>
-      <c r="AP2" s="117"/>
-      <c r="AQ2" s="117"/>
-      <c r="AR2" s="117"/>
-      <c r="AS2" s="110">
+      <c r="AO2" s="144"/>
+      <c r="AP2" s="144"/>
+      <c r="AQ2" s="144"/>
+      <c r="AR2" s="144"/>
+      <c r="AS2" s="111">
         <v>45707</v>
       </c>
-      <c r="AT2" s="111"/>
-      <c r="AU2" s="111"/>
-      <c r="AV2" s="111"/>
-      <c r="AW2" s="112"/>
-      <c r="AX2" s="120" t="s">
+      <c r="AT2" s="112"/>
+      <c r="AU2" s="112"/>
+      <c r="AV2" s="112"/>
+      <c r="AW2" s="113"/>
+      <c r="AX2" s="117" t="s">
         <v>56</v>
       </c>
-      <c r="AY2" s="120"/>
-      <c r="AZ2" s="120"/>
-      <c r="BA2" s="120"/>
-      <c r="BB2" s="120"/>
-      <c r="BC2" s="110">
+      <c r="AY2" s="117"/>
+      <c r="AZ2" s="117"/>
+      <c r="BA2" s="117"/>
+      <c r="BB2" s="117"/>
+      <c r="BC2" s="111">
         <v>45701</v>
       </c>
-      <c r="BD2" s="111"/>
-      <c r="BE2" s="111"/>
-      <c r="BF2" s="111"/>
-      <c r="BG2" s="112"/>
-      <c r="BH2" s="120" t="s">
+      <c r="BD2" s="112"/>
+      <c r="BE2" s="112"/>
+      <c r="BF2" s="112"/>
+      <c r="BG2" s="113"/>
+      <c r="BH2" s="117" t="s">
         <v>56</v>
       </c>
-      <c r="BI2" s="120"/>
-      <c r="BJ2" s="120"/>
-      <c r="BK2" s="120"/>
-      <c r="BL2" s="120"/>
+      <c r="BI2" s="117"/>
+      <c r="BJ2" s="117"/>
+      <c r="BK2" s="117"/>
+      <c r="BL2" s="117"/>
       <c r="BM2" s="2"/>
     </row>
     <row r="3" spans="1:65" s="5" customFormat="1" ht="10.5" customHeight="1">
-      <c r="A3" s="145"/>
-      <c r="B3" s="146"/>
-      <c r="C3" s="146"/>
-      <c r="D3" s="146"/>
-      <c r="E3" s="147"/>
-      <c r="F3" s="145"/>
-      <c r="G3" s="146"/>
-      <c r="H3" s="146"/>
-      <c r="I3" s="146"/>
-      <c r="J3" s="147"/>
-      <c r="K3" s="108"/>
-      <c r="L3" s="108"/>
-      <c r="M3" s="108"/>
-      <c r="N3" s="108"/>
-      <c r="O3" s="109"/>
-      <c r="P3" s="107"/>
-      <c r="Q3" s="108"/>
-      <c r="R3" s="108"/>
-      <c r="S3" s="108"/>
-      <c r="T3" s="109"/>
-      <c r="U3" s="107"/>
-      <c r="V3" s="108"/>
-      <c r="W3" s="108"/>
-      <c r="X3" s="108"/>
-      <c r="Y3" s="108"/>
-      <c r="Z3" s="108"/>
-      <c r="AA3" s="108"/>
-      <c r="AB3" s="108"/>
-      <c r="AC3" s="108"/>
-      <c r="AD3" s="108"/>
-      <c r="AE3" s="108"/>
-      <c r="AF3" s="108"/>
-      <c r="AG3" s="108"/>
-      <c r="AH3" s="109"/>
-      <c r="AI3" s="113"/>
-      <c r="AJ3" s="114"/>
-      <c r="AK3" s="114"/>
-      <c r="AL3" s="114"/>
-      <c r="AM3" s="115"/>
-      <c r="AN3" s="118"/>
-      <c r="AO3" s="119"/>
-      <c r="AP3" s="119"/>
-      <c r="AQ3" s="119"/>
-      <c r="AR3" s="119"/>
-      <c r="AS3" s="113"/>
-      <c r="AT3" s="114"/>
-      <c r="AU3" s="114"/>
-      <c r="AV3" s="114"/>
-      <c r="AW3" s="115"/>
-      <c r="AX3" s="120"/>
-      <c r="AY3" s="120"/>
-      <c r="AZ3" s="120"/>
-      <c r="BA3" s="120"/>
-      <c r="BB3" s="120"/>
-      <c r="BC3" s="113"/>
-      <c r="BD3" s="114"/>
-      <c r="BE3" s="114"/>
-      <c r="BF3" s="114"/>
-      <c r="BG3" s="115"/>
-      <c r="BH3" s="120"/>
-      <c r="BI3" s="120"/>
-      <c r="BJ3" s="120"/>
-      <c r="BK3" s="120"/>
-      <c r="BL3" s="120"/>
+      <c r="A3" s="126"/>
+      <c r="B3" s="127"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="127"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="127"/>
+      <c r="H3" s="127"/>
+      <c r="I3" s="127"/>
+      <c r="J3" s="128"/>
+      <c r="K3" s="131"/>
+      <c r="L3" s="131"/>
+      <c r="M3" s="131"/>
+      <c r="N3" s="131"/>
+      <c r="O3" s="132"/>
+      <c r="P3" s="143"/>
+      <c r="Q3" s="131"/>
+      <c r="R3" s="131"/>
+      <c r="S3" s="131"/>
+      <c r="T3" s="132"/>
+      <c r="U3" s="143"/>
+      <c r="V3" s="131"/>
+      <c r="W3" s="131"/>
+      <c r="X3" s="131"/>
+      <c r="Y3" s="131"/>
+      <c r="Z3" s="131"/>
+      <c r="AA3" s="131"/>
+      <c r="AB3" s="131"/>
+      <c r="AC3" s="131"/>
+      <c r="AD3" s="131"/>
+      <c r="AE3" s="131"/>
+      <c r="AF3" s="131"/>
+      <c r="AG3" s="131"/>
+      <c r="AH3" s="132"/>
+      <c r="AI3" s="114"/>
+      <c r="AJ3" s="115"/>
+      <c r="AK3" s="115"/>
+      <c r="AL3" s="115"/>
+      <c r="AM3" s="116"/>
+      <c r="AN3" s="145"/>
+      <c r="AO3" s="146"/>
+      <c r="AP3" s="146"/>
+      <c r="AQ3" s="146"/>
+      <c r="AR3" s="146"/>
+      <c r="AS3" s="114"/>
+      <c r="AT3" s="115"/>
+      <c r="AU3" s="115"/>
+      <c r="AV3" s="115"/>
+      <c r="AW3" s="116"/>
+      <c r="AX3" s="117"/>
+      <c r="AY3" s="117"/>
+      <c r="AZ3" s="117"/>
+      <c r="BA3" s="117"/>
+      <c r="BB3" s="117"/>
+      <c r="BC3" s="114"/>
+      <c r="BD3" s="115"/>
+      <c r="BE3" s="115"/>
+      <c r="BF3" s="115"/>
+      <c r="BG3" s="116"/>
+      <c r="BH3" s="117"/>
+      <c r="BI3" s="117"/>
+      <c r="BJ3" s="117"/>
+      <c r="BK3" s="117"/>
+      <c r="BL3" s="117"/>
       <c r="BM3" s="2"/>
     </row>
     <row r="4" spans="1:65" s="5" customFormat="1" ht="9.75" customHeight="1">
@@ -3660,6 +3714,523 @@
       <c r="BL8" s="15"/>
     </row>
     <row r="9" spans="1:65">
+      <c r="B9" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="22">
+    <mergeCell ref="AI2:AM3"/>
+    <mergeCell ref="AN2:AR3"/>
+    <mergeCell ref="AS2:AW3"/>
+    <mergeCell ref="AX2:BB3"/>
+    <mergeCell ref="BC2:BG3"/>
+    <mergeCell ref="BH2:BL3"/>
+    <mergeCell ref="AN1:AR1"/>
+    <mergeCell ref="AS1:AW1"/>
+    <mergeCell ref="AX1:BB1"/>
+    <mergeCell ref="BC1:BG1"/>
+    <mergeCell ref="BH1:BL1"/>
+    <mergeCell ref="A2:E3"/>
+    <mergeCell ref="F2:J3"/>
+    <mergeCell ref="K2:O3"/>
+    <mergeCell ref="P2:T3"/>
+    <mergeCell ref="U2:AH3"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="P1:T1"/>
+    <mergeCell ref="U1:AH1"/>
+    <mergeCell ref="AI1:AM1"/>
+  </mergeCells>
+  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="91" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;P/&amp;N</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:BM25"/>
+  <sheetFormatPr defaultColWidth="2.33203125" defaultRowHeight="13.8"/>
+  <cols>
+    <col min="1" max="2" width="3.109375" style="2" customWidth="1"/>
+    <col min="3" max="5" width="2.77734375" style="2" customWidth="1"/>
+    <col min="6" max="7" width="2.33203125" style="2"/>
+    <col min="8" max="8" width="2.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="3" style="2" customWidth="1"/>
+    <col min="10" max="10" width="3.44140625" style="2" customWidth="1"/>
+    <col min="11" max="46" width="2.33203125" style="2"/>
+    <col min="47" max="47" width="2.88671875" style="2" customWidth="1"/>
+    <col min="48" max="48" width="2.6640625" style="2" customWidth="1"/>
+    <col min="49" max="49" width="2.77734375" style="2" customWidth="1"/>
+    <col min="50" max="16384" width="2.33203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:65" s="5" customFormat="1">
+      <c r="A1" s="107" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="107" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="119" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="109"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="120" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="121"/>
+      <c r="R1" s="121"/>
+      <c r="S1" s="121"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="120" t="s">
+        <v>15</v>
+      </c>
+      <c r="V1" s="121"/>
+      <c r="W1" s="121"/>
+      <c r="X1" s="121"/>
+      <c r="Y1" s="121"/>
+      <c r="Z1" s="121"/>
+      <c r="AA1" s="121"/>
+      <c r="AB1" s="121"/>
+      <c r="AC1" s="121"/>
+      <c r="AD1" s="121"/>
+      <c r="AE1" s="121"/>
+      <c r="AF1" s="121"/>
+      <c r="AG1" s="121"/>
+      <c r="AH1" s="122"/>
+      <c r="AI1" s="133" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ1" s="134"/>
+      <c r="AK1" s="134"/>
+      <c r="AL1" s="134"/>
+      <c r="AM1" s="135"/>
+      <c r="AN1" s="133" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO1" s="134"/>
+      <c r="AP1" s="134"/>
+      <c r="AQ1" s="134"/>
+      <c r="AR1" s="135"/>
+      <c r="AS1" s="133" t="s">
+        <v>18</v>
+      </c>
+      <c r="AT1" s="134"/>
+      <c r="AU1" s="134"/>
+      <c r="AV1" s="134"/>
+      <c r="AW1" s="135"/>
+      <c r="AX1" s="107" t="s">
+        <v>19</v>
+      </c>
+      <c r="AY1" s="109"/>
+      <c r="AZ1" s="109"/>
+      <c r="BA1" s="109"/>
+      <c r="BB1" s="110"/>
+      <c r="BC1" s="107" t="s">
+        <v>20</v>
+      </c>
+      <c r="BD1" s="108"/>
+      <c r="BE1" s="108"/>
+      <c r="BF1" s="109"/>
+      <c r="BG1" s="110"/>
+      <c r="BH1" s="103" t="s">
+        <v>21</v>
+      </c>
+      <c r="BI1" s="104"/>
+      <c r="BJ1" s="105"/>
+      <c r="BK1" s="105"/>
+      <c r="BL1" s="106"/>
+      <c r="BM1" s="2"/>
+    </row>
+    <row r="2" spans="1:65" s="5" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A2" s="123" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="124"/>
+      <c r="C2" s="124"/>
+      <c r="D2" s="124"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="123" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2" s="124"/>
+      <c r="H2" s="124"/>
+      <c r="I2" s="124"/>
+      <c r="J2" s="125"/>
+      <c r="K2" s="129" t="s">
+        <v>54</v>
+      </c>
+      <c r="L2" s="129"/>
+      <c r="M2" s="129"/>
+      <c r="N2" s="129"/>
+      <c r="O2" s="130"/>
+      <c r="P2" s="142" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q2" s="129"/>
+      <c r="R2" s="129"/>
+      <c r="S2" s="129"/>
+      <c r="T2" s="130"/>
+      <c r="U2" s="142" t="s">
+        <v>52</v>
+      </c>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
+      <c r="X2" s="129"/>
+      <c r="Y2" s="129"/>
+      <c r="Z2" s="129"/>
+      <c r="AA2" s="129"/>
+      <c r="AB2" s="129"/>
+      <c r="AC2" s="129"/>
+      <c r="AD2" s="129"/>
+      <c r="AE2" s="129"/>
+      <c r="AF2" s="129"/>
+      <c r="AG2" s="129"/>
+      <c r="AH2" s="130"/>
+      <c r="AI2" s="111">
+        <v>45701</v>
+      </c>
+      <c r="AJ2" s="112"/>
+      <c r="AK2" s="112"/>
+      <c r="AL2" s="112"/>
+      <c r="AM2" s="113"/>
+      <c r="AN2" s="123" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO2" s="144"/>
+      <c r="AP2" s="144"/>
+      <c r="AQ2" s="144"/>
+      <c r="AR2" s="144"/>
+      <c r="AS2" s="111">
+        <v>45707</v>
+      </c>
+      <c r="AT2" s="112"/>
+      <c r="AU2" s="112"/>
+      <c r="AV2" s="112"/>
+      <c r="AW2" s="113"/>
+      <c r="AX2" s="117" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY2" s="117"/>
+      <c r="AZ2" s="117"/>
+      <c r="BA2" s="117"/>
+      <c r="BB2" s="117"/>
+      <c r="BC2" s="111">
+        <v>45701</v>
+      </c>
+      <c r="BD2" s="112"/>
+      <c r="BE2" s="112"/>
+      <c r="BF2" s="112"/>
+      <c r="BG2" s="113"/>
+      <c r="BH2" s="117" t="s">
+        <v>56</v>
+      </c>
+      <c r="BI2" s="117"/>
+      <c r="BJ2" s="117"/>
+      <c r="BK2" s="117"/>
+      <c r="BL2" s="117"/>
+      <c r="BM2" s="2"/>
+    </row>
+    <row r="3" spans="1:65" s="5" customFormat="1" ht="10.5" customHeight="1">
+      <c r="A3" s="126"/>
+      <c r="B3" s="127"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="127"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="127"/>
+      <c r="H3" s="127"/>
+      <c r="I3" s="127"/>
+      <c r="J3" s="128"/>
+      <c r="K3" s="131"/>
+      <c r="L3" s="131"/>
+      <c r="M3" s="131"/>
+      <c r="N3" s="131"/>
+      <c r="O3" s="132"/>
+      <c r="P3" s="143"/>
+      <c r="Q3" s="131"/>
+      <c r="R3" s="131"/>
+      <c r="S3" s="131"/>
+      <c r="T3" s="132"/>
+      <c r="U3" s="143"/>
+      <c r="V3" s="131"/>
+      <c r="W3" s="131"/>
+      <c r="X3" s="131"/>
+      <c r="Y3" s="131"/>
+      <c r="Z3" s="131"/>
+      <c r="AA3" s="131"/>
+      <c r="AB3" s="131"/>
+      <c r="AC3" s="131"/>
+      <c r="AD3" s="131"/>
+      <c r="AE3" s="131"/>
+      <c r="AF3" s="131"/>
+      <c r="AG3" s="131"/>
+      <c r="AH3" s="132"/>
+      <c r="AI3" s="114"/>
+      <c r="AJ3" s="115"/>
+      <c r="AK3" s="115"/>
+      <c r="AL3" s="115"/>
+      <c r="AM3" s="116"/>
+      <c r="AN3" s="145"/>
+      <c r="AO3" s="146"/>
+      <c r="AP3" s="146"/>
+      <c r="AQ3" s="146"/>
+      <c r="AR3" s="146"/>
+      <c r="AS3" s="114"/>
+      <c r="AT3" s="115"/>
+      <c r="AU3" s="115"/>
+      <c r="AV3" s="115"/>
+      <c r="AW3" s="116"/>
+      <c r="AX3" s="117"/>
+      <c r="AY3" s="117"/>
+      <c r="AZ3" s="117"/>
+      <c r="BA3" s="117"/>
+      <c r="BB3" s="117"/>
+      <c r="BC3" s="114"/>
+      <c r="BD3" s="115"/>
+      <c r="BE3" s="115"/>
+      <c r="BF3" s="115"/>
+      <c r="BG3" s="116"/>
+      <c r="BH3" s="117"/>
+      <c r="BI3" s="117"/>
+      <c r="BJ3" s="117"/>
+      <c r="BK3" s="117"/>
+      <c r="BL3" s="117"/>
+      <c r="BM3" s="2"/>
+    </row>
+    <row r="4" spans="1:65" s="5" customFormat="1" ht="9.75" customHeight="1">
+      <c r="A4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="42"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="42"/>
+      <c r="N4" s="42"/>
+      <c r="O4" s="42"/>
+      <c r="P4" s="42"/>
+      <c r="Q4" s="42"/>
+      <c r="R4" s="42"/>
+      <c r="S4" s="42"/>
+      <c r="T4" s="42"/>
+      <c r="U4" s="42"/>
+      <c r="V4" s="42"/>
+      <c r="W4" s="42"/>
+      <c r="X4" s="42"/>
+      <c r="Y4" s="42"/>
+      <c r="Z4" s="42"/>
+      <c r="AA4" s="42"/>
+      <c r="AB4" s="42"/>
+      <c r="AC4" s="42"/>
+      <c r="AD4" s="42"/>
+      <c r="AE4" s="42"/>
+      <c r="AF4" s="42"/>
+      <c r="AG4" s="42"/>
+      <c r="AH4" s="42"/>
+      <c r="AI4" s="44"/>
+      <c r="AJ4" s="42"/>
+      <c r="AK4" s="42"/>
+      <c r="AL4" s="42"/>
+      <c r="AM4" s="42"/>
+      <c r="AN4" s="47"/>
+      <c r="AO4" s="43"/>
+      <c r="AP4" s="43"/>
+      <c r="AQ4" s="43"/>
+      <c r="AR4" s="43"/>
+      <c r="AS4" s="44"/>
+      <c r="AT4" s="42"/>
+      <c r="AU4" s="42"/>
+      <c r="AV4" s="42"/>
+      <c r="AW4" s="42"/>
+      <c r="AX4" s="52"/>
+      <c r="AY4" s="52"/>
+      <c r="AZ4" s="52"/>
+      <c r="BA4" s="52"/>
+      <c r="BB4" s="52"/>
+      <c r="BC4" s="44"/>
+      <c r="BD4" s="44"/>
+      <c r="BE4" s="44"/>
+      <c r="BF4" s="44"/>
+      <c r="BG4" s="44"/>
+      <c r="BH4" s="47"/>
+      <c r="BI4" s="47"/>
+      <c r="BJ4" s="43"/>
+      <c r="BK4" s="43"/>
+      <c r="BL4" s="45"/>
+      <c r="BM4" s="2"/>
+    </row>
+    <row r="5" spans="1:65">
+      <c r="A5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="10"/>
+      <c r="X5" s="10"/>
+      <c r="Y5" s="10"/>
+      <c r="Z5" s="10"/>
+      <c r="AA5" s="10"/>
+      <c r="AB5" s="10"/>
+      <c r="AC5" s="10"/>
+      <c r="AD5" s="10"/>
+      <c r="AE5" s="10"/>
+      <c r="AF5" s="10"/>
+      <c r="AG5" s="10"/>
+      <c r="AH5" s="10"/>
+      <c r="AI5" s="10"/>
+      <c r="AJ5" s="10"/>
+      <c r="AK5" s="10"/>
+      <c r="AL5" s="10"/>
+      <c r="AM5" s="10"/>
+      <c r="AN5" s="10"/>
+      <c r="AO5" s="10"/>
+      <c r="AP5" s="10"/>
+      <c r="AQ5" s="10"/>
+      <c r="AR5" s="10"/>
+      <c r="AS5" s="10"/>
+      <c r="AT5" s="10"/>
+      <c r="AU5" s="10"/>
+      <c r="AV5" s="10"/>
+      <c r="AW5" s="10"/>
+      <c r="AX5" s="10"/>
+      <c r="AY5" s="10"/>
+      <c r="AZ5" s="10"/>
+      <c r="BA5" s="10"/>
+      <c r="BB5" s="10"/>
+      <c r="BC5" s="10"/>
+      <c r="BD5" s="10"/>
+      <c r="BE5" s="10"/>
+      <c r="BF5" s="10"/>
+      <c r="BG5" s="10"/>
+      <c r="BH5" s="10"/>
+      <c r="BI5" s="10"/>
+      <c r="BJ5" s="10"/>
+      <c r="BK5" s="10"/>
+      <c r="BL5" s="11"/>
+    </row>
+    <row r="6" spans="1:65">
+      <c r="A6" s="13"/>
+      <c r="BL6" s="3"/>
+    </row>
+    <row r="7" spans="1:65">
+      <c r="A7" s="13"/>
+      <c r="B7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="BL7" s="3"/>
+    </row>
+    <row r="8" spans="1:65">
+      <c r="A8" s="14"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12"/>
+      <c r="T8" s="12"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="12"/>
+      <c r="W8" s="12"/>
+      <c r="X8" s="12"/>
+      <c r="Y8" s="12"/>
+      <c r="Z8" s="12"/>
+      <c r="AA8" s="12"/>
+      <c r="AB8" s="12"/>
+      <c r="AC8" s="12"/>
+      <c r="AD8" s="12"/>
+      <c r="AE8" s="12"/>
+      <c r="AF8" s="12"/>
+      <c r="AG8" s="12"/>
+      <c r="AH8" s="12"/>
+      <c r="AI8" s="12"/>
+      <c r="AJ8" s="12"/>
+      <c r="AK8" s="12"/>
+      <c r="AL8" s="12"/>
+      <c r="AM8" s="12"/>
+      <c r="AN8" s="12"/>
+      <c r="AO8" s="12"/>
+      <c r="AP8" s="12"/>
+      <c r="AQ8" s="12"/>
+      <c r="AR8" s="12"/>
+      <c r="AS8" s="12"/>
+      <c r="AT8" s="12"/>
+      <c r="AU8" s="12"/>
+      <c r="AV8" s="12"/>
+      <c r="AW8" s="12"/>
+      <c r="AX8" s="12"/>
+      <c r="AY8" s="12"/>
+      <c r="AZ8" s="12"/>
+      <c r="BA8" s="12"/>
+      <c r="BB8" s="12"/>
+      <c r="BC8" s="12"/>
+      <c r="BD8" s="12"/>
+      <c r="BE8" s="12"/>
+      <c r="BF8" s="12"/>
+      <c r="BG8" s="12"/>
+      <c r="BH8" s="12"/>
+      <c r="BI8" s="12"/>
+      <c r="BJ8" s="12"/>
+      <c r="BK8" s="12"/>
+      <c r="BL8" s="15"/>
+    </row>
+    <row r="9" spans="1:65">
       <c r="A9" s="6"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -3701,23 +4272,23 @@
         <v>24</v>
       </c>
       <c r="AN10" s="19"/>
-      <c r="AO10" s="121" t="s">
+      <c r="AO10" s="136" t="s">
         <v>28</v>
       </c>
-      <c r="AP10" s="122"/>
-      <c r="AQ10" s="122"/>
-      <c r="AR10" s="122"/>
-      <c r="AS10" s="122"/>
-      <c r="AT10" s="122"/>
-      <c r="AU10" s="122"/>
-      <c r="AV10" s="122"/>
-      <c r="AW10" s="122"/>
-      <c r="AX10" s="122"/>
-      <c r="AY10" s="122"/>
-      <c r="AZ10" s="122"/>
-      <c r="BA10" s="122"/>
-      <c r="BB10" s="122"/>
-      <c r="BC10" s="123"/>
+      <c r="AP10" s="137"/>
+      <c r="AQ10" s="137"/>
+      <c r="AR10" s="137"/>
+      <c r="AS10" s="137"/>
+      <c r="AT10" s="137"/>
+      <c r="AU10" s="137"/>
+      <c r="AV10" s="137"/>
+      <c r="AW10" s="137"/>
+      <c r="AX10" s="137"/>
+      <c r="AY10" s="137"/>
+      <c r="AZ10" s="137"/>
+      <c r="BA10" s="137"/>
+      <c r="BB10" s="137"/>
+      <c r="BC10" s="138"/>
       <c r="BD10" s="21" t="s">
         <v>5</v>
       </c>
@@ -3727,31 +4298,31 @@
     </row>
     <row r="11" spans="1:65" ht="15" customHeight="1">
       <c r="A11" s="13"/>
-      <c r="AM11" s="100" t="s">
+      <c r="AM11" s="147" t="s">
         <v>2</v>
       </c>
-      <c r="AN11" s="101"/>
-      <c r="AO11" s="124" t="s">
+      <c r="AN11" s="148"/>
+      <c r="AO11" s="100" t="s">
         <v>49</v>
       </c>
-      <c r="AP11" s="125"/>
-      <c r="AQ11" s="125"/>
-      <c r="AR11" s="125"/>
-      <c r="AS11" s="125"/>
-      <c r="AT11" s="125"/>
-      <c r="AU11" s="125"/>
-      <c r="AV11" s="125"/>
-      <c r="AW11" s="125"/>
-      <c r="AX11" s="125"/>
-      <c r="AY11" s="125"/>
-      <c r="AZ11" s="125"/>
-      <c r="BA11" s="125"/>
-      <c r="BB11" s="125"/>
-      <c r="BC11" s="126"/>
-      <c r="BD11" s="102" t="s">
+      <c r="AP11" s="101"/>
+      <c r="AQ11" s="101"/>
+      <c r="AR11" s="101"/>
+      <c r="AS11" s="101"/>
+      <c r="AT11" s="101"/>
+      <c r="AU11" s="101"/>
+      <c r="AV11" s="101"/>
+      <c r="AW11" s="101"/>
+      <c r="AX11" s="101"/>
+      <c r="AY11" s="101"/>
+      <c r="AZ11" s="101"/>
+      <c r="BA11" s="101"/>
+      <c r="BB11" s="101"/>
+      <c r="BC11" s="102"/>
+      <c r="BD11" s="149" t="s">
         <v>47</v>
       </c>
-      <c r="BE11" s="103"/>
+      <c r="BE11" s="150"/>
       <c r="BF11" s="13"/>
       <c r="BL11" s="3"/>
     </row>
@@ -3760,61 +4331,61 @@
       <c r="B12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="AM12" s="100" t="s">
+      <c r="AM12" s="147" t="s">
         <v>6</v>
       </c>
-      <c r="AN12" s="101"/>
-      <c r="AO12" s="127" t="s">
+      <c r="AN12" s="148"/>
+      <c r="AO12" s="139" t="s">
         <v>50</v>
       </c>
-      <c r="AP12" s="128"/>
-      <c r="AQ12" s="128"/>
-      <c r="AR12" s="128"/>
-      <c r="AS12" s="128"/>
-      <c r="AT12" s="128"/>
-      <c r="AU12" s="128"/>
-      <c r="AV12" s="128"/>
-      <c r="AW12" s="128"/>
-      <c r="AX12" s="128"/>
-      <c r="AY12" s="128"/>
-      <c r="AZ12" s="128"/>
-      <c r="BA12" s="128"/>
-      <c r="BB12" s="128"/>
-      <c r="BC12" s="129"/>
-      <c r="BD12" s="102" t="s">
+      <c r="AP12" s="140"/>
+      <c r="AQ12" s="140"/>
+      <c r="AR12" s="140"/>
+      <c r="AS12" s="140"/>
+      <c r="AT12" s="140"/>
+      <c r="AU12" s="140"/>
+      <c r="AV12" s="140"/>
+      <c r="AW12" s="140"/>
+      <c r="AX12" s="140"/>
+      <c r="AY12" s="140"/>
+      <c r="AZ12" s="140"/>
+      <c r="BA12" s="140"/>
+      <c r="BB12" s="140"/>
+      <c r="BC12" s="141"/>
+      <c r="BD12" s="149" t="s">
         <v>42</v>
       </c>
-      <c r="BE12" s="103"/>
+      <c r="BE12" s="150"/>
       <c r="BF12" s="13"/>
       <c r="BL12" s="3"/>
     </row>
     <row r="13" spans="1:65" ht="15" customHeight="1">
       <c r="A13" s="13"/>
-      <c r="AM13" s="100" t="s">
+      <c r="AM13" s="147" t="s">
         <v>3</v>
       </c>
-      <c r="AN13" s="101"/>
-      <c r="AO13" s="127" t="s">
+      <c r="AN13" s="148"/>
+      <c r="AO13" s="139" t="s">
         <v>51</v>
       </c>
-      <c r="AP13" s="128"/>
-      <c r="AQ13" s="128"/>
-      <c r="AR13" s="128"/>
-      <c r="AS13" s="128"/>
-      <c r="AT13" s="128"/>
-      <c r="AU13" s="128"/>
-      <c r="AV13" s="128"/>
-      <c r="AW13" s="128"/>
-      <c r="AX13" s="128"/>
-      <c r="AY13" s="128"/>
-      <c r="AZ13" s="128"/>
-      <c r="BA13" s="128"/>
-      <c r="BB13" s="128"/>
-      <c r="BC13" s="129"/>
-      <c r="BD13" s="102" t="s">
+      <c r="AP13" s="140"/>
+      <c r="AQ13" s="140"/>
+      <c r="AR13" s="140"/>
+      <c r="AS13" s="140"/>
+      <c r="AT13" s="140"/>
+      <c r="AU13" s="140"/>
+      <c r="AV13" s="140"/>
+      <c r="AW13" s="140"/>
+      <c r="AX13" s="140"/>
+      <c r="AY13" s="140"/>
+      <c r="AZ13" s="140"/>
+      <c r="BA13" s="140"/>
+      <c r="BB13" s="140"/>
+      <c r="BC13" s="141"/>
+      <c r="BD13" s="149" t="s">
         <v>42</v>
       </c>
-      <c r="BE13" s="103"/>
+      <c r="BE13" s="150"/>
       <c r="BF13" s="13"/>
       <c r="BL13" s="3"/>
     </row>
@@ -3822,21 +4393,21 @@
       <c r="A14" s="13"/>
       <c r="AM14" s="27"/>
       <c r="AN14" s="28"/>
-      <c r="AO14" s="124"/>
-      <c r="AP14" s="125"/>
-      <c r="AQ14" s="125"/>
-      <c r="AR14" s="125"/>
-      <c r="AS14" s="125"/>
-      <c r="AT14" s="125"/>
-      <c r="AU14" s="125"/>
-      <c r="AV14" s="125"/>
-      <c r="AW14" s="125"/>
-      <c r="AX14" s="125"/>
-      <c r="AY14" s="125"/>
-      <c r="AZ14" s="125"/>
-      <c r="BA14" s="125"/>
-      <c r="BB14" s="125"/>
-      <c r="BC14" s="126"/>
+      <c r="AO14" s="100"/>
+      <c r="AP14" s="101"/>
+      <c r="AQ14" s="101"/>
+      <c r="AR14" s="101"/>
+      <c r="AS14" s="101"/>
+      <c r="AT14" s="101"/>
+      <c r="AU14" s="101"/>
+      <c r="AV14" s="101"/>
+      <c r="AW14" s="101"/>
+      <c r="AX14" s="101"/>
+      <c r="AY14" s="101"/>
+      <c r="AZ14" s="101"/>
+      <c r="BA14" s="101"/>
+      <c r="BB14" s="101"/>
+      <c r="BC14" s="102"/>
       <c r="BD14" s="31"/>
       <c r="BE14" s="32"/>
       <c r="BF14" s="13"/>
@@ -3846,21 +4417,21 @@
       <c r="A15" s="13"/>
       <c r="AM15" s="27"/>
       <c r="AN15" s="28"/>
-      <c r="AO15" s="124"/>
-      <c r="AP15" s="125"/>
-      <c r="AQ15" s="125"/>
-      <c r="AR15" s="125"/>
-      <c r="AS15" s="125"/>
-      <c r="AT15" s="125"/>
-      <c r="AU15" s="125"/>
-      <c r="AV15" s="125"/>
-      <c r="AW15" s="125"/>
-      <c r="AX15" s="125"/>
-      <c r="AY15" s="125"/>
-      <c r="AZ15" s="125"/>
-      <c r="BA15" s="125"/>
-      <c r="BB15" s="125"/>
-      <c r="BC15" s="126"/>
+      <c r="AO15" s="100"/>
+      <c r="AP15" s="101"/>
+      <c r="AQ15" s="101"/>
+      <c r="AR15" s="101"/>
+      <c r="AS15" s="101"/>
+      <c r="AT15" s="101"/>
+      <c r="AU15" s="101"/>
+      <c r="AV15" s="101"/>
+      <c r="AW15" s="101"/>
+      <c r="AX15" s="101"/>
+      <c r="AY15" s="101"/>
+      <c r="AZ15" s="101"/>
+      <c r="BA15" s="101"/>
+      <c r="BB15" s="101"/>
+      <c r="BC15" s="102"/>
       <c r="BD15" s="31"/>
       <c r="BE15" s="32"/>
       <c r="BF15" s="13"/>
@@ -3870,21 +4441,21 @@
       <c r="A16" s="13"/>
       <c r="AM16" s="27"/>
       <c r="AN16" s="28"/>
-      <c r="AO16" s="124"/>
-      <c r="AP16" s="125"/>
-      <c r="AQ16" s="125"/>
-      <c r="AR16" s="125"/>
-      <c r="AS16" s="125"/>
-      <c r="AT16" s="125"/>
-      <c r="AU16" s="125"/>
-      <c r="AV16" s="125"/>
-      <c r="AW16" s="125"/>
-      <c r="AX16" s="125"/>
-      <c r="AY16" s="125"/>
-      <c r="AZ16" s="125"/>
-      <c r="BA16" s="125"/>
-      <c r="BB16" s="125"/>
-      <c r="BC16" s="126"/>
+      <c r="AO16" s="100"/>
+      <c r="AP16" s="101"/>
+      <c r="AQ16" s="101"/>
+      <c r="AR16" s="101"/>
+      <c r="AS16" s="101"/>
+      <c r="AT16" s="101"/>
+      <c r="AU16" s="101"/>
+      <c r="AV16" s="101"/>
+      <c r="AW16" s="101"/>
+      <c r="AX16" s="101"/>
+      <c r="AY16" s="101"/>
+      <c r="AZ16" s="101"/>
+      <c r="BA16" s="101"/>
+      <c r="BB16" s="101"/>
+      <c r="BC16" s="102"/>
       <c r="BD16" s="31"/>
       <c r="BE16" s="32"/>
       <c r="BF16" s="13"/>
@@ -3894,21 +4465,21 @@
       <c r="A17" s="13"/>
       <c r="AM17" s="27"/>
       <c r="AN17" s="28"/>
-      <c r="AO17" s="124"/>
-      <c r="AP17" s="125"/>
-      <c r="AQ17" s="125"/>
-      <c r="AR17" s="125"/>
-      <c r="AS17" s="125"/>
-      <c r="AT17" s="125"/>
-      <c r="AU17" s="125"/>
-      <c r="AV17" s="125"/>
-      <c r="AW17" s="125"/>
-      <c r="AX17" s="125"/>
-      <c r="AY17" s="125"/>
-      <c r="AZ17" s="125"/>
-      <c r="BA17" s="125"/>
-      <c r="BB17" s="125"/>
-      <c r="BC17" s="126"/>
+      <c r="AO17" s="100"/>
+      <c r="AP17" s="101"/>
+      <c r="AQ17" s="101"/>
+      <c r="AR17" s="101"/>
+      <c r="AS17" s="101"/>
+      <c r="AT17" s="101"/>
+      <c r="AU17" s="101"/>
+      <c r="AV17" s="101"/>
+      <c r="AW17" s="101"/>
+      <c r="AX17" s="101"/>
+      <c r="AY17" s="101"/>
+      <c r="AZ17" s="101"/>
+      <c r="BA17" s="101"/>
+      <c r="BB17" s="101"/>
+      <c r="BC17" s="102"/>
       <c r="BD17" s="31"/>
       <c r="BE17" s="32"/>
       <c r="BF17" s="13"/>
@@ -3918,21 +4489,21 @@
       <c r="A18" s="13"/>
       <c r="AM18" s="27"/>
       <c r="AN18" s="28"/>
-      <c r="AO18" s="124"/>
-      <c r="AP18" s="125"/>
-      <c r="AQ18" s="125"/>
-      <c r="AR18" s="125"/>
-      <c r="AS18" s="125"/>
-      <c r="AT18" s="125"/>
-      <c r="AU18" s="125"/>
-      <c r="AV18" s="125"/>
-      <c r="AW18" s="125"/>
-      <c r="AX18" s="125"/>
-      <c r="AY18" s="125"/>
-      <c r="AZ18" s="125"/>
-      <c r="BA18" s="125"/>
-      <c r="BB18" s="125"/>
-      <c r="BC18" s="126"/>
+      <c r="AO18" s="100"/>
+      <c r="AP18" s="101"/>
+      <c r="AQ18" s="101"/>
+      <c r="AR18" s="101"/>
+      <c r="AS18" s="101"/>
+      <c r="AT18" s="101"/>
+      <c r="AU18" s="101"/>
+      <c r="AV18" s="101"/>
+      <c r="AW18" s="101"/>
+      <c r="AX18" s="101"/>
+      <c r="AY18" s="101"/>
+      <c r="AZ18" s="101"/>
+      <c r="BA18" s="101"/>
+      <c r="BB18" s="101"/>
+      <c r="BC18" s="102"/>
       <c r="BD18" s="34"/>
       <c r="BE18" s="35"/>
       <c r="BF18" s="13"/>
@@ -4124,11 +4695,22 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="AO14:BC14"/>
-    <mergeCell ref="AO18:BC18"/>
-    <mergeCell ref="AO15:BC15"/>
-    <mergeCell ref="AO16:BC16"/>
-    <mergeCell ref="AO17:BC17"/>
+    <mergeCell ref="AM11:AN11"/>
+    <mergeCell ref="BD11:BE11"/>
+    <mergeCell ref="AM12:AN12"/>
+    <mergeCell ref="BD12:BE12"/>
+    <mergeCell ref="AM13:AN13"/>
+    <mergeCell ref="BD13:BE13"/>
+    <mergeCell ref="P2:T3"/>
+    <mergeCell ref="U2:AH3"/>
+    <mergeCell ref="AI2:AM3"/>
+    <mergeCell ref="AN2:AR3"/>
+    <mergeCell ref="AS2:AW3"/>
+    <mergeCell ref="AX2:BB3"/>
+    <mergeCell ref="AO10:BC10"/>
+    <mergeCell ref="AO11:BC11"/>
+    <mergeCell ref="AO12:BC12"/>
+    <mergeCell ref="AO13:BC13"/>
     <mergeCell ref="BH1:BL1"/>
     <mergeCell ref="BC1:BG1"/>
     <mergeCell ref="BC2:BG3"/>
@@ -4145,22 +4727,11 @@
     <mergeCell ref="AN1:AR1"/>
     <mergeCell ref="AS1:AW1"/>
     <mergeCell ref="AX1:BB1"/>
-    <mergeCell ref="AX2:BB3"/>
-    <mergeCell ref="AO10:BC10"/>
-    <mergeCell ref="AO11:BC11"/>
-    <mergeCell ref="AO12:BC12"/>
-    <mergeCell ref="AO13:BC13"/>
-    <mergeCell ref="P2:T3"/>
-    <mergeCell ref="U2:AH3"/>
-    <mergeCell ref="AI2:AM3"/>
-    <mergeCell ref="AN2:AR3"/>
-    <mergeCell ref="AS2:AW3"/>
-    <mergeCell ref="AM11:AN11"/>
-    <mergeCell ref="BD11:BE11"/>
-    <mergeCell ref="AM12:AN12"/>
-    <mergeCell ref="BD12:BE12"/>
-    <mergeCell ref="AM13:AN13"/>
-    <mergeCell ref="BD13:BE13"/>
+    <mergeCell ref="AO14:BC14"/>
+    <mergeCell ref="AO18:BC18"/>
+    <mergeCell ref="AO15:BC15"/>
+    <mergeCell ref="AO16:BC16"/>
+    <mergeCell ref="AO17:BC17"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="91" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4171,7 +4742,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4193,182 +4764,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:60" s="5" customFormat="1" ht="15" customHeight="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="134" t="s">
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="139" t="s">
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="119" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="136"/>
-      <c r="M1" s="136"/>
-      <c r="N1" s="136"/>
-      <c r="O1" s="137"/>
-      <c r="P1" s="140" t="s">
+      <c r="L1" s="109"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="120" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="141"/>
-      <c r="R1" s="141"/>
-      <c r="S1" s="141"/>
-      <c r="T1" s="142"/>
-      <c r="U1" s="140" t="s">
+      <c r="Q1" s="121"/>
+      <c r="R1" s="121"/>
+      <c r="S1" s="121"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="120" t="s">
         <v>15</v>
       </c>
-      <c r="V1" s="141"/>
-      <c r="W1" s="141"/>
-      <c r="X1" s="141"/>
-      <c r="Y1" s="141"/>
-      <c r="Z1" s="141"/>
-      <c r="AA1" s="141"/>
-      <c r="AB1" s="141"/>
-      <c r="AC1" s="141"/>
-      <c r="AD1" s="142"/>
-      <c r="AE1" s="148" t="s">
+      <c r="V1" s="121"/>
+      <c r="W1" s="121"/>
+      <c r="X1" s="121"/>
+      <c r="Y1" s="121"/>
+      <c r="Z1" s="121"/>
+      <c r="AA1" s="121"/>
+      <c r="AB1" s="121"/>
+      <c r="AC1" s="121"/>
+      <c r="AD1" s="122"/>
+      <c r="AE1" s="133" t="s">
         <v>16</v>
       </c>
-      <c r="AF1" s="149"/>
-      <c r="AG1" s="149"/>
-      <c r="AH1" s="149"/>
-      <c r="AI1" s="150"/>
-      <c r="AJ1" s="148" t="s">
+      <c r="AF1" s="134"/>
+      <c r="AG1" s="134"/>
+      <c r="AH1" s="134"/>
+      <c r="AI1" s="135"/>
+      <c r="AJ1" s="133" t="s">
         <v>17</v>
       </c>
-      <c r="AK1" s="149"/>
-      <c r="AL1" s="149"/>
-      <c r="AM1" s="150"/>
-      <c r="AN1" s="148" t="s">
+      <c r="AK1" s="134"/>
+      <c r="AL1" s="134"/>
+      <c r="AM1" s="135"/>
+      <c r="AN1" s="133" t="s">
         <v>18</v>
       </c>
-      <c r="AO1" s="149"/>
-      <c r="AP1" s="149"/>
-      <c r="AQ1" s="149"/>
-      <c r="AR1" s="150"/>
-      <c r="AS1" s="134" t="s">
+      <c r="AO1" s="134"/>
+      <c r="AP1" s="134"/>
+      <c r="AQ1" s="134"/>
+      <c r="AR1" s="135"/>
+      <c r="AS1" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="AT1" s="136"/>
-      <c r="AU1" s="136"/>
-      <c r="AV1" s="136"/>
-      <c r="AW1" s="137"/>
-      <c r="AX1" s="134" t="s">
+      <c r="AT1" s="109"/>
+      <c r="AU1" s="109"/>
+      <c r="AV1" s="109"/>
+      <c r="AW1" s="110"/>
+      <c r="AX1" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="AY1" s="135"/>
-      <c r="AZ1" s="135"/>
-      <c r="BA1" s="136"/>
-      <c r="BB1" s="137"/>
-      <c r="BC1" s="130" t="s">
+      <c r="AY1" s="108"/>
+      <c r="AZ1" s="108"/>
+      <c r="BA1" s="109"/>
+      <c r="BB1" s="110"/>
+      <c r="BC1" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="BD1" s="131"/>
-      <c r="BE1" s="132"/>
-      <c r="BF1" s="132"/>
-      <c r="BG1" s="133"/>
+      <c r="BD1" s="104"/>
+      <c r="BE1" s="105"/>
+      <c r="BF1" s="105"/>
+      <c r="BG1" s="106"/>
       <c r="BH1" s="2"/>
     </row>
     <row r="2" spans="1:60" s="5" customFormat="1" ht="29.25" customHeight="1">
-      <c r="A2" s="151" t="str">
+      <c r="A2" s="154" t="str">
         <f>Overview!A2</f>
         <v>EduLearn</v>
       </c>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
-      <c r="E2" s="153"/>
-      <c r="F2" s="151" t="str">
+      <c r="B2" s="155"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="154" t="str">
         <f>Overview!F2</f>
         <v>Courses</v>
       </c>
-      <c r="G2" s="152"/>
-      <c r="H2" s="152"/>
-      <c r="I2" s="152"/>
-      <c r="J2" s="153"/>
-      <c r="K2" s="154" t="str">
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
+      <c r="J2" s="156"/>
+      <c r="K2" s="157" t="str">
         <f>Overview!K2</f>
         <v>SC001</v>
       </c>
-      <c r="L2" s="154"/>
-      <c r="M2" s="154"/>
-      <c r="N2" s="154"/>
-      <c r="O2" s="155"/>
-      <c r="P2" s="156" t="str">
+      <c r="L2" s="157"/>
+      <c r="M2" s="157"/>
+      <c r="N2" s="157"/>
+      <c r="O2" s="158"/>
+      <c r="P2" s="159" t="str">
         <f>Overview!P2</f>
         <v>SC Name</v>
       </c>
-      <c r="Q2" s="154"/>
-      <c r="R2" s="154"/>
-      <c r="S2" s="154"/>
-      <c r="T2" s="155"/>
-      <c r="U2" s="156" t="str">
+      <c r="Q2" s="157"/>
+      <c r="R2" s="157"/>
+      <c r="S2" s="157"/>
+      <c r="T2" s="158"/>
+      <c r="U2" s="159" t="str">
         <f>Overview!U2</f>
         <v>Template_DD_v1.0.xlsx</v>
       </c>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
-      <c r="Z2" s="154"/>
-      <c r="AA2" s="154"/>
-      <c r="AB2" s="154"/>
-      <c r="AC2" s="154"/>
-      <c r="AD2" s="155"/>
-      <c r="AE2" s="157">
+      <c r="V2" s="157"/>
+      <c r="W2" s="157"/>
+      <c r="X2" s="157"/>
+      <c r="Y2" s="157"/>
+      <c r="Z2" s="157"/>
+      <c r="AA2" s="157"/>
+      <c r="AB2" s="157"/>
+      <c r="AC2" s="157"/>
+      <c r="AD2" s="158"/>
+      <c r="AE2" s="151">
         <f>Overview!AI2</f>
         <v>45701</v>
       </c>
-      <c r="AF2" s="158"/>
-      <c r="AG2" s="158"/>
-      <c r="AH2" s="158"/>
-      <c r="AI2" s="159"/>
-      <c r="AJ2" s="151" t="str">
+      <c r="AF2" s="152"/>
+      <c r="AG2" s="152"/>
+      <c r="AH2" s="152"/>
+      <c r="AI2" s="153"/>
+      <c r="AJ2" s="154" t="str">
         <f>Overview!AN2</f>
         <v>BangNT</v>
       </c>
-      <c r="AK2" s="152"/>
-      <c r="AL2" s="152"/>
-      <c r="AM2" s="152"/>
-      <c r="AN2" s="157">
+      <c r="AK2" s="155"/>
+      <c r="AL2" s="155"/>
+      <c r="AM2" s="155"/>
+      <c r="AN2" s="151">
         <f>Overview!AS2</f>
         <v>45707</v>
       </c>
-      <c r="AO2" s="158"/>
-      <c r="AP2" s="158"/>
-      <c r="AQ2" s="158"/>
-      <c r="AR2" s="159"/>
-      <c r="AS2" s="120" t="str">
+      <c r="AO2" s="152"/>
+      <c r="AP2" s="152"/>
+      <c r="AQ2" s="152"/>
+      <c r="AR2" s="153"/>
+      <c r="AS2" s="117" t="str">
         <f>Overview!AX2</f>
         <v>BangNT</v>
       </c>
-      <c r="AT2" s="120"/>
-      <c r="AU2" s="120"/>
-      <c r="AV2" s="120"/>
-      <c r="AW2" s="120"/>
-      <c r="AX2" s="157">
+      <c r="AT2" s="117"/>
+      <c r="AU2" s="117"/>
+      <c r="AV2" s="117"/>
+      <c r="AW2" s="117"/>
+      <c r="AX2" s="151">
         <f>Overview!BC2</f>
         <v>45701</v>
       </c>
-      <c r="AY2" s="158"/>
-      <c r="AZ2" s="158"/>
-      <c r="BA2" s="158"/>
-      <c r="BB2" s="159"/>
-      <c r="BC2" s="151" t="str">
+      <c r="AY2" s="152"/>
+      <c r="AZ2" s="152"/>
+      <c r="BA2" s="152"/>
+      <c r="BB2" s="153"/>
+      <c r="BC2" s="154" t="str">
         <f>Overview!BH2</f>
         <v>BangNT</v>
       </c>
-      <c r="BD2" s="152"/>
-      <c r="BE2" s="152"/>
-      <c r="BF2" s="152"/>
-      <c r="BG2" s="153"/>
+      <c r="BD2" s="155"/>
+      <c r="BE2" s="155"/>
+      <c r="BF2" s="155"/>
+      <c r="BG2" s="156"/>
       <c r="BH2" s="2"/>
     </row>
     <row r="3" spans="1:60" s="4" customFormat="1" ht="10.5" customHeight="1">
@@ -4625,28 +5196,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="AE2:AI2"/>
-    <mergeCell ref="AJ2:AM2"/>
-    <mergeCell ref="AN2:AR2"/>
-    <mergeCell ref="AS2:AW2"/>
-    <mergeCell ref="AX2:BB2"/>
+    <mergeCell ref="AE1:AI1"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="P1:T1"/>
+    <mergeCell ref="U1:AD1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="K2:O2"/>
+    <mergeCell ref="P2:T2"/>
+    <mergeCell ref="U2:AD2"/>
     <mergeCell ref="BC2:BG2"/>
     <mergeCell ref="AJ1:AM1"/>
     <mergeCell ref="AN1:AR1"/>
     <mergeCell ref="AS1:AW1"/>
     <mergeCell ref="AX1:BB1"/>
     <mergeCell ref="BC1:BG1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="K2:O2"/>
-    <mergeCell ref="P2:T2"/>
-    <mergeCell ref="U2:AD2"/>
-    <mergeCell ref="AE1:AI1"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:O1"/>
-    <mergeCell ref="P1:T1"/>
-    <mergeCell ref="U1:AD1"/>
+    <mergeCell ref="AE2:AI2"/>
+    <mergeCell ref="AJ2:AM2"/>
+    <mergeCell ref="AN2:AR2"/>
+    <mergeCell ref="AS2:AW2"/>
+    <mergeCell ref="AX2:BB2"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="98" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -4656,7 +5227,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{567342E5-F899-48BD-974B-0DC0FF996026}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4678,182 +5249,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:60" s="5" customFormat="1" ht="15" customHeight="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="134" t="s">
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="139" t="s">
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="119" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="136"/>
-      <c r="M1" s="136"/>
-      <c r="N1" s="136"/>
-      <c r="O1" s="137"/>
-      <c r="P1" s="140" t="s">
+      <c r="L1" s="109"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="120" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="141"/>
-      <c r="R1" s="141"/>
-      <c r="S1" s="141"/>
-      <c r="T1" s="142"/>
-      <c r="U1" s="140" t="s">
+      <c r="Q1" s="121"/>
+      <c r="R1" s="121"/>
+      <c r="S1" s="121"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="120" t="s">
         <v>15</v>
       </c>
-      <c r="V1" s="141"/>
-      <c r="W1" s="141"/>
-      <c r="X1" s="141"/>
-      <c r="Y1" s="141"/>
-      <c r="Z1" s="141"/>
-      <c r="AA1" s="141"/>
-      <c r="AB1" s="141"/>
-      <c r="AC1" s="141"/>
-      <c r="AD1" s="142"/>
-      <c r="AE1" s="148" t="s">
+      <c r="V1" s="121"/>
+      <c r="W1" s="121"/>
+      <c r="X1" s="121"/>
+      <c r="Y1" s="121"/>
+      <c r="Z1" s="121"/>
+      <c r="AA1" s="121"/>
+      <c r="AB1" s="121"/>
+      <c r="AC1" s="121"/>
+      <c r="AD1" s="122"/>
+      <c r="AE1" s="133" t="s">
         <v>16</v>
       </c>
-      <c r="AF1" s="149"/>
-      <c r="AG1" s="149"/>
-      <c r="AH1" s="149"/>
-      <c r="AI1" s="150"/>
-      <c r="AJ1" s="148" t="s">
+      <c r="AF1" s="134"/>
+      <c r="AG1" s="134"/>
+      <c r="AH1" s="134"/>
+      <c r="AI1" s="135"/>
+      <c r="AJ1" s="133" t="s">
         <v>17</v>
       </c>
-      <c r="AK1" s="149"/>
-      <c r="AL1" s="149"/>
-      <c r="AM1" s="150"/>
-      <c r="AN1" s="148" t="s">
+      <c r="AK1" s="134"/>
+      <c r="AL1" s="134"/>
+      <c r="AM1" s="135"/>
+      <c r="AN1" s="133" t="s">
         <v>18</v>
       </c>
-      <c r="AO1" s="149"/>
-      <c r="AP1" s="149"/>
-      <c r="AQ1" s="149"/>
-      <c r="AR1" s="150"/>
-      <c r="AS1" s="134" t="s">
+      <c r="AO1" s="134"/>
+      <c r="AP1" s="134"/>
+      <c r="AQ1" s="134"/>
+      <c r="AR1" s="135"/>
+      <c r="AS1" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="AT1" s="136"/>
-      <c r="AU1" s="136"/>
-      <c r="AV1" s="136"/>
-      <c r="AW1" s="137"/>
-      <c r="AX1" s="134" t="s">
+      <c r="AT1" s="109"/>
+      <c r="AU1" s="109"/>
+      <c r="AV1" s="109"/>
+      <c r="AW1" s="110"/>
+      <c r="AX1" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="AY1" s="135"/>
-      <c r="AZ1" s="135"/>
-      <c r="BA1" s="136"/>
-      <c r="BB1" s="137"/>
-      <c r="BC1" s="130" t="s">
+      <c r="AY1" s="108"/>
+      <c r="AZ1" s="108"/>
+      <c r="BA1" s="109"/>
+      <c r="BB1" s="110"/>
+      <c r="BC1" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="BD1" s="131"/>
-      <c r="BE1" s="132"/>
-      <c r="BF1" s="132"/>
-      <c r="BG1" s="133"/>
+      <c r="BD1" s="104"/>
+      <c r="BE1" s="105"/>
+      <c r="BF1" s="105"/>
+      <c r="BG1" s="106"/>
       <c r="BH1" s="2"/>
     </row>
     <row r="2" spans="1:60" s="5" customFormat="1" ht="29.25" customHeight="1">
-      <c r="A2" s="151" t="str">
+      <c r="A2" s="154" t="str">
         <f>Overview!A2</f>
         <v>EduLearn</v>
       </c>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
-      <c r="E2" s="153"/>
-      <c r="F2" s="151" t="str">
+      <c r="B2" s="155"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="154" t="str">
         <f>Overview!F2</f>
         <v>Courses</v>
       </c>
-      <c r="G2" s="152"/>
-      <c r="H2" s="152"/>
-      <c r="I2" s="152"/>
-      <c r="J2" s="153"/>
-      <c r="K2" s="154" t="str">
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
+      <c r="J2" s="156"/>
+      <c r="K2" s="157" t="str">
         <f>Overview!K2</f>
         <v>SC001</v>
       </c>
-      <c r="L2" s="154"/>
-      <c r="M2" s="154"/>
-      <c r="N2" s="154"/>
-      <c r="O2" s="155"/>
-      <c r="P2" s="156" t="str">
+      <c r="L2" s="157"/>
+      <c r="M2" s="157"/>
+      <c r="N2" s="157"/>
+      <c r="O2" s="158"/>
+      <c r="P2" s="159" t="str">
         <f>Overview!P2</f>
         <v>SC Name</v>
       </c>
-      <c r="Q2" s="154"/>
-      <c r="R2" s="154"/>
-      <c r="S2" s="154"/>
-      <c r="T2" s="155"/>
-      <c r="U2" s="156" t="str">
+      <c r="Q2" s="157"/>
+      <c r="R2" s="157"/>
+      <c r="S2" s="157"/>
+      <c r="T2" s="158"/>
+      <c r="U2" s="159" t="str">
         <f>Overview!U2</f>
         <v>Template_DD_v1.0.xlsx</v>
       </c>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
-      <c r="Z2" s="154"/>
-      <c r="AA2" s="154"/>
-      <c r="AB2" s="154"/>
-      <c r="AC2" s="154"/>
-      <c r="AD2" s="155"/>
-      <c r="AE2" s="157">
+      <c r="V2" s="157"/>
+      <c r="W2" s="157"/>
+      <c r="X2" s="157"/>
+      <c r="Y2" s="157"/>
+      <c r="Z2" s="157"/>
+      <c r="AA2" s="157"/>
+      <c r="AB2" s="157"/>
+      <c r="AC2" s="157"/>
+      <c r="AD2" s="158"/>
+      <c r="AE2" s="151">
         <f>Overview!AI2</f>
         <v>45701</v>
       </c>
-      <c r="AF2" s="158"/>
-      <c r="AG2" s="158"/>
-      <c r="AH2" s="158"/>
-      <c r="AI2" s="159"/>
-      <c r="AJ2" s="151" t="str">
+      <c r="AF2" s="152"/>
+      <c r="AG2" s="152"/>
+      <c r="AH2" s="152"/>
+      <c r="AI2" s="153"/>
+      <c r="AJ2" s="154" t="str">
         <f>Overview!AN2</f>
         <v>BangNT</v>
       </c>
-      <c r="AK2" s="152"/>
-      <c r="AL2" s="152"/>
-      <c r="AM2" s="152"/>
-      <c r="AN2" s="157">
+      <c r="AK2" s="155"/>
+      <c r="AL2" s="155"/>
+      <c r="AM2" s="155"/>
+      <c r="AN2" s="151">
         <f>Overview!AS2</f>
         <v>45707</v>
       </c>
-      <c r="AO2" s="158"/>
-      <c r="AP2" s="158"/>
-      <c r="AQ2" s="158"/>
-      <c r="AR2" s="159"/>
-      <c r="AS2" s="120" t="str">
+      <c r="AO2" s="152"/>
+      <c r="AP2" s="152"/>
+      <c r="AQ2" s="152"/>
+      <c r="AR2" s="153"/>
+      <c r="AS2" s="117" t="str">
         <f>Overview!AX2</f>
         <v>BangNT</v>
       </c>
-      <c r="AT2" s="120"/>
-      <c r="AU2" s="120"/>
-      <c r="AV2" s="120"/>
-      <c r="AW2" s="120"/>
-      <c r="AX2" s="157">
+      <c r="AT2" s="117"/>
+      <c r="AU2" s="117"/>
+      <c r="AV2" s="117"/>
+      <c r="AW2" s="117"/>
+      <c r="AX2" s="151">
         <f>Overview!BC2</f>
         <v>45701</v>
       </c>
-      <c r="AY2" s="158"/>
-      <c r="AZ2" s="158"/>
-      <c r="BA2" s="158"/>
-      <c r="BB2" s="159"/>
-      <c r="BC2" s="151" t="str">
+      <c r="AY2" s="152"/>
+      <c r="AZ2" s="152"/>
+      <c r="BA2" s="152"/>
+      <c r="BB2" s="153"/>
+      <c r="BC2" s="154" t="str">
         <f>Overview!BH2</f>
         <v>BangNT</v>
       </c>
-      <c r="BD2" s="152"/>
-      <c r="BE2" s="152"/>
-      <c r="BF2" s="152"/>
-      <c r="BG2" s="153"/>
+      <c r="BD2" s="155"/>
+      <c r="BE2" s="155"/>
+      <c r="BF2" s="155"/>
+      <c r="BG2" s="156"/>
       <c r="BH2" s="2"/>
     </row>
     <row r="3" spans="1:60" s="4" customFormat="1" ht="10.5" customHeight="1">
@@ -5050,28 +5621,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="AE2:AI2"/>
+    <mergeCell ref="AJ2:AM2"/>
+    <mergeCell ref="AN2:AR2"/>
+    <mergeCell ref="AS2:AW2"/>
+    <mergeCell ref="AX2:BB2"/>
+    <mergeCell ref="BC2:BG2"/>
+    <mergeCell ref="AJ1:AM1"/>
+    <mergeCell ref="AN1:AR1"/>
+    <mergeCell ref="AS1:AW1"/>
+    <mergeCell ref="AX1:BB1"/>
+    <mergeCell ref="BC1:BG1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="K2:O2"/>
+    <mergeCell ref="P2:T2"/>
+    <mergeCell ref="U2:AD2"/>
     <mergeCell ref="AE1:AI1"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="F1:J1"/>
     <mergeCell ref="K1:O1"/>
     <mergeCell ref="P1:T1"/>
     <mergeCell ref="U1:AD1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="K2:O2"/>
-    <mergeCell ref="P2:T2"/>
-    <mergeCell ref="U2:AD2"/>
-    <mergeCell ref="BC2:BG2"/>
-    <mergeCell ref="AJ1:AM1"/>
-    <mergeCell ref="AN1:AR1"/>
-    <mergeCell ref="AS1:AW1"/>
-    <mergeCell ref="AX1:BB1"/>
-    <mergeCell ref="BC1:BG1"/>
-    <mergeCell ref="AE2:AI2"/>
-    <mergeCell ref="AJ2:AM2"/>
-    <mergeCell ref="AN2:AR2"/>
-    <mergeCell ref="AS2:AW2"/>
-    <mergeCell ref="AX2:BB2"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="98" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -5082,7 +5653,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46B661F1-2324-49A4-A317-7CE94BF662B6}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -5104,182 +5675,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:60" s="5" customFormat="1" ht="15" customHeight="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="134" t="s">
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="139" t="s">
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="119" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="136"/>
-      <c r="M1" s="136"/>
-      <c r="N1" s="136"/>
-      <c r="O1" s="137"/>
-      <c r="P1" s="140" t="s">
+      <c r="L1" s="109"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="120" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="141"/>
-      <c r="R1" s="141"/>
-      <c r="S1" s="141"/>
-      <c r="T1" s="142"/>
-      <c r="U1" s="140" t="s">
+      <c r="Q1" s="121"/>
+      <c r="R1" s="121"/>
+      <c r="S1" s="121"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="120" t="s">
         <v>15</v>
       </c>
-      <c r="V1" s="141"/>
-      <c r="W1" s="141"/>
-      <c r="X1" s="141"/>
-      <c r="Y1" s="141"/>
-      <c r="Z1" s="141"/>
-      <c r="AA1" s="141"/>
-      <c r="AB1" s="141"/>
-      <c r="AC1" s="141"/>
-      <c r="AD1" s="142"/>
-      <c r="AE1" s="148" t="s">
+      <c r="V1" s="121"/>
+      <c r="W1" s="121"/>
+      <c r="X1" s="121"/>
+      <c r="Y1" s="121"/>
+      <c r="Z1" s="121"/>
+      <c r="AA1" s="121"/>
+      <c r="AB1" s="121"/>
+      <c r="AC1" s="121"/>
+      <c r="AD1" s="122"/>
+      <c r="AE1" s="133" t="s">
         <v>16</v>
       </c>
-      <c r="AF1" s="149"/>
-      <c r="AG1" s="149"/>
-      <c r="AH1" s="149"/>
-      <c r="AI1" s="150"/>
-      <c r="AJ1" s="148" t="s">
+      <c r="AF1" s="134"/>
+      <c r="AG1" s="134"/>
+      <c r="AH1" s="134"/>
+      <c r="AI1" s="135"/>
+      <c r="AJ1" s="133" t="s">
         <v>17</v>
       </c>
-      <c r="AK1" s="149"/>
-      <c r="AL1" s="149"/>
-      <c r="AM1" s="150"/>
-      <c r="AN1" s="148" t="s">
+      <c r="AK1" s="134"/>
+      <c r="AL1" s="134"/>
+      <c r="AM1" s="135"/>
+      <c r="AN1" s="133" t="s">
         <v>18</v>
       </c>
-      <c r="AO1" s="149"/>
-      <c r="AP1" s="149"/>
-      <c r="AQ1" s="149"/>
-      <c r="AR1" s="150"/>
-      <c r="AS1" s="134" t="s">
+      <c r="AO1" s="134"/>
+      <c r="AP1" s="134"/>
+      <c r="AQ1" s="134"/>
+      <c r="AR1" s="135"/>
+      <c r="AS1" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="AT1" s="136"/>
-      <c r="AU1" s="136"/>
-      <c r="AV1" s="136"/>
-      <c r="AW1" s="137"/>
-      <c r="AX1" s="134" t="s">
+      <c r="AT1" s="109"/>
+      <c r="AU1" s="109"/>
+      <c r="AV1" s="109"/>
+      <c r="AW1" s="110"/>
+      <c r="AX1" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="AY1" s="135"/>
-      <c r="AZ1" s="135"/>
-      <c r="BA1" s="136"/>
-      <c r="BB1" s="137"/>
-      <c r="BC1" s="130" t="s">
+      <c r="AY1" s="108"/>
+      <c r="AZ1" s="108"/>
+      <c r="BA1" s="109"/>
+      <c r="BB1" s="110"/>
+      <c r="BC1" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="BD1" s="131"/>
-      <c r="BE1" s="132"/>
-      <c r="BF1" s="132"/>
-      <c r="BG1" s="133"/>
+      <c r="BD1" s="104"/>
+      <c r="BE1" s="105"/>
+      <c r="BF1" s="105"/>
+      <c r="BG1" s="106"/>
       <c r="BH1" s="2"/>
     </row>
     <row r="2" spans="1:60" s="5" customFormat="1" ht="29.25" customHeight="1">
-      <c r="A2" s="151" t="str">
+      <c r="A2" s="154" t="str">
         <f>Overview!A2</f>
         <v>EduLearn</v>
       </c>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
-      <c r="E2" s="153"/>
-      <c r="F2" s="151" t="str">
+      <c r="B2" s="155"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="154" t="str">
         <f>Overview!F2</f>
         <v>Courses</v>
       </c>
-      <c r="G2" s="152"/>
-      <c r="H2" s="152"/>
-      <c r="I2" s="152"/>
-      <c r="J2" s="153"/>
-      <c r="K2" s="154" t="str">
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
+      <c r="J2" s="156"/>
+      <c r="K2" s="157" t="str">
         <f>Overview!K2</f>
         <v>SC001</v>
       </c>
-      <c r="L2" s="154"/>
-      <c r="M2" s="154"/>
-      <c r="N2" s="154"/>
-      <c r="O2" s="155"/>
-      <c r="P2" s="156" t="str">
+      <c r="L2" s="157"/>
+      <c r="M2" s="157"/>
+      <c r="N2" s="157"/>
+      <c r="O2" s="158"/>
+      <c r="P2" s="159" t="str">
         <f>Overview!P2</f>
         <v>SC Name</v>
       </c>
-      <c r="Q2" s="154"/>
-      <c r="R2" s="154"/>
-      <c r="S2" s="154"/>
-      <c r="T2" s="155"/>
-      <c r="U2" s="156" t="str">
+      <c r="Q2" s="157"/>
+      <c r="R2" s="157"/>
+      <c r="S2" s="157"/>
+      <c r="T2" s="158"/>
+      <c r="U2" s="159" t="str">
         <f>Overview!U2</f>
         <v>Template_DD_v1.0.xlsx</v>
       </c>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
-      <c r="Z2" s="154"/>
-      <c r="AA2" s="154"/>
-      <c r="AB2" s="154"/>
-      <c r="AC2" s="154"/>
-      <c r="AD2" s="155"/>
-      <c r="AE2" s="157">
+      <c r="V2" s="157"/>
+      <c r="W2" s="157"/>
+      <c r="X2" s="157"/>
+      <c r="Y2" s="157"/>
+      <c r="Z2" s="157"/>
+      <c r="AA2" s="157"/>
+      <c r="AB2" s="157"/>
+      <c r="AC2" s="157"/>
+      <c r="AD2" s="158"/>
+      <c r="AE2" s="151">
         <f>Overview!AI2</f>
         <v>45701</v>
       </c>
-      <c r="AF2" s="158"/>
-      <c r="AG2" s="158"/>
-      <c r="AH2" s="158"/>
-      <c r="AI2" s="159"/>
-      <c r="AJ2" s="151" t="str">
+      <c r="AF2" s="152"/>
+      <c r="AG2" s="152"/>
+      <c r="AH2" s="152"/>
+      <c r="AI2" s="153"/>
+      <c r="AJ2" s="154" t="str">
         <f>Overview!AN2</f>
         <v>BangNT</v>
       </c>
-      <c r="AK2" s="152"/>
-      <c r="AL2" s="152"/>
-      <c r="AM2" s="152"/>
-      <c r="AN2" s="157">
+      <c r="AK2" s="155"/>
+      <c r="AL2" s="155"/>
+      <c r="AM2" s="155"/>
+      <c r="AN2" s="151">
         <f>Overview!AS2</f>
         <v>45707</v>
       </c>
-      <c r="AO2" s="158"/>
-      <c r="AP2" s="158"/>
-      <c r="AQ2" s="158"/>
-      <c r="AR2" s="159"/>
-      <c r="AS2" s="120" t="str">
+      <c r="AO2" s="152"/>
+      <c r="AP2" s="152"/>
+      <c r="AQ2" s="152"/>
+      <c r="AR2" s="153"/>
+      <c r="AS2" s="117" t="str">
         <f>Overview!AX2</f>
         <v>BangNT</v>
       </c>
-      <c r="AT2" s="120"/>
-      <c r="AU2" s="120"/>
-      <c r="AV2" s="120"/>
-      <c r="AW2" s="120"/>
-      <c r="AX2" s="157">
+      <c r="AT2" s="117"/>
+      <c r="AU2" s="117"/>
+      <c r="AV2" s="117"/>
+      <c r="AW2" s="117"/>
+      <c r="AX2" s="151">
         <f>Overview!BC2</f>
         <v>45701</v>
       </c>
-      <c r="AY2" s="158"/>
-      <c r="AZ2" s="158"/>
-      <c r="BA2" s="158"/>
-      <c r="BB2" s="159"/>
-      <c r="BC2" s="151" t="str">
+      <c r="AY2" s="152"/>
+      <c r="AZ2" s="152"/>
+      <c r="BA2" s="152"/>
+      <c r="BB2" s="153"/>
+      <c r="BC2" s="154" t="str">
         <f>Overview!BH2</f>
         <v>BangNT</v>
       </c>
-      <c r="BD2" s="152"/>
-      <c r="BE2" s="152"/>
-      <c r="BF2" s="152"/>
-      <c r="BG2" s="153"/>
+      <c r="BD2" s="155"/>
+      <c r="BE2" s="155"/>
+      <c r="BF2" s="155"/>
+      <c r="BG2" s="156"/>
       <c r="BH2" s="2"/>
     </row>
     <row r="3" spans="1:60" s="4" customFormat="1" ht="10.5" customHeight="1">
@@ -5476,28 +6047,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="AE2:AI2"/>
+    <mergeCell ref="AJ2:AM2"/>
+    <mergeCell ref="AN2:AR2"/>
+    <mergeCell ref="AS2:AW2"/>
+    <mergeCell ref="AX2:BB2"/>
+    <mergeCell ref="BC2:BG2"/>
+    <mergeCell ref="AJ1:AM1"/>
+    <mergeCell ref="AN1:AR1"/>
+    <mergeCell ref="AS1:AW1"/>
+    <mergeCell ref="AX1:BB1"/>
+    <mergeCell ref="BC1:BG1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="K2:O2"/>
+    <mergeCell ref="P2:T2"/>
+    <mergeCell ref="U2:AD2"/>
     <mergeCell ref="AE1:AI1"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="F1:J1"/>
     <mergeCell ref="K1:O1"/>
     <mergeCell ref="P1:T1"/>
     <mergeCell ref="U1:AD1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="K2:O2"/>
-    <mergeCell ref="P2:T2"/>
-    <mergeCell ref="U2:AD2"/>
-    <mergeCell ref="BC2:BG2"/>
-    <mergeCell ref="AJ1:AM1"/>
-    <mergeCell ref="AN1:AR1"/>
-    <mergeCell ref="AS1:AW1"/>
-    <mergeCell ref="AX1:BB1"/>
-    <mergeCell ref="BC1:BG1"/>
-    <mergeCell ref="AE2:AI2"/>
-    <mergeCell ref="AJ2:AM2"/>
-    <mergeCell ref="AN2:AR2"/>
-    <mergeCell ref="AS2:AW2"/>
-    <mergeCell ref="AX2:BB2"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="98" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -5508,7 +6079,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -5534,207 +6105,207 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:72" s="5" customFormat="1" ht="15" customHeight="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="134" t="s">
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="139" t="s">
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="119" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="136"/>
-      <c r="M1" s="136"/>
-      <c r="N1" s="136"/>
-      <c r="O1" s="137"/>
-      <c r="P1" s="140" t="s">
+      <c r="L1" s="109"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="120" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="141"/>
-      <c r="R1" s="141"/>
-      <c r="S1" s="141"/>
-      <c r="T1" s="142"/>
-      <c r="U1" s="140" t="s">
+      <c r="Q1" s="121"/>
+      <c r="R1" s="121"/>
+      <c r="S1" s="121"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="120" t="s">
         <v>15</v>
       </c>
-      <c r="V1" s="141"/>
-      <c r="W1" s="141"/>
-      <c r="X1" s="141"/>
-      <c r="Y1" s="141"/>
-      <c r="Z1" s="141"/>
-      <c r="AA1" s="141"/>
-      <c r="AB1" s="141"/>
-      <c r="AC1" s="141"/>
-      <c r="AD1" s="142"/>
-      <c r="AE1" s="148" t="s">
+      <c r="V1" s="121"/>
+      <c r="W1" s="121"/>
+      <c r="X1" s="121"/>
+      <c r="Y1" s="121"/>
+      <c r="Z1" s="121"/>
+      <c r="AA1" s="121"/>
+      <c r="AB1" s="121"/>
+      <c r="AC1" s="121"/>
+      <c r="AD1" s="122"/>
+      <c r="AE1" s="133" t="s">
         <v>16</v>
       </c>
-      <c r="AF1" s="149"/>
-      <c r="AG1" s="149"/>
-      <c r="AH1" s="149"/>
-      <c r="AI1" s="150"/>
-      <c r="AJ1" s="148" t="s">
+      <c r="AF1" s="134"/>
+      <c r="AG1" s="134"/>
+      <c r="AH1" s="134"/>
+      <c r="AI1" s="135"/>
+      <c r="AJ1" s="133" t="s">
         <v>17</v>
       </c>
-      <c r="AK1" s="149"/>
-      <c r="AL1" s="149"/>
-      <c r="AM1" s="150"/>
-      <c r="AN1" s="148" t="s">
+      <c r="AK1" s="134"/>
+      <c r="AL1" s="134"/>
+      <c r="AM1" s="135"/>
+      <c r="AN1" s="133" t="s">
         <v>18</v>
       </c>
-      <c r="AO1" s="149"/>
-      <c r="AP1" s="149"/>
-      <c r="AQ1" s="149"/>
-      <c r="AR1" s="150"/>
-      <c r="AS1" s="134" t="s">
+      <c r="AO1" s="134"/>
+      <c r="AP1" s="134"/>
+      <c r="AQ1" s="134"/>
+      <c r="AR1" s="135"/>
+      <c r="AS1" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="AT1" s="136"/>
-      <c r="AU1" s="136"/>
-      <c r="AV1" s="136"/>
-      <c r="AW1" s="137"/>
-      <c r="AX1" s="134" t="s">
+      <c r="AT1" s="109"/>
+      <c r="AU1" s="109"/>
+      <c r="AV1" s="109"/>
+      <c r="AW1" s="110"/>
+      <c r="AX1" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="AY1" s="135"/>
-      <c r="AZ1" s="135"/>
-      <c r="BA1" s="136"/>
-      <c r="BB1" s="137"/>
-      <c r="BC1" s="174" t="s">
+      <c r="AY1" s="108"/>
+      <c r="AZ1" s="108"/>
+      <c r="BA1" s="109"/>
+      <c r="BB1" s="110"/>
+      <c r="BC1" s="168" t="s">
         <v>21</v>
       </c>
-      <c r="BD1" s="175"/>
-      <c r="BE1" s="175"/>
-      <c r="BF1" s="175"/>
-      <c r="BG1" s="175"/>
-      <c r="BH1" s="175"/>
-      <c r="BI1" s="175"/>
-      <c r="BJ1" s="175"/>
-      <c r="BK1" s="175"/>
-      <c r="BL1" s="175"/>
-      <c r="BM1" s="175"/>
-      <c r="BN1" s="175"/>
-      <c r="BO1" s="175"/>
-      <c r="BP1" s="175"/>
-      <c r="BQ1" s="175"/>
-      <c r="BR1" s="175"/>
-      <c r="BS1" s="175"/>
-      <c r="BT1" s="175"/>
+      <c r="BD1" s="169"/>
+      <c r="BE1" s="169"/>
+      <c r="BF1" s="169"/>
+      <c r="BG1" s="169"/>
+      <c r="BH1" s="169"/>
+      <c r="BI1" s="169"/>
+      <c r="BJ1" s="169"/>
+      <c r="BK1" s="169"/>
+      <c r="BL1" s="169"/>
+      <c r="BM1" s="169"/>
+      <c r="BN1" s="169"/>
+      <c r="BO1" s="169"/>
+      <c r="BP1" s="169"/>
+      <c r="BQ1" s="169"/>
+      <c r="BR1" s="169"/>
+      <c r="BS1" s="169"/>
+      <c r="BT1" s="169"/>
     </row>
     <row r="2" spans="1:72" s="5" customFormat="1" ht="29.25" customHeight="1">
-      <c r="A2" s="151" t="str">
+      <c r="A2" s="154" t="str">
         <f>Overview!A2</f>
         <v>EduLearn</v>
       </c>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
-      <c r="E2" s="153"/>
-      <c r="F2" s="151" t="str">
+      <c r="B2" s="155"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="154" t="str">
         <f>Overview!F2</f>
         <v>Courses</v>
       </c>
-      <c r="G2" s="152"/>
-      <c r="H2" s="152"/>
-      <c r="I2" s="152"/>
-      <c r="J2" s="153"/>
-      <c r="K2" s="154" t="str">
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
+      <c r="J2" s="156"/>
+      <c r="K2" s="157" t="str">
         <f>Overview!K2</f>
         <v>SC001</v>
       </c>
-      <c r="L2" s="154"/>
-      <c r="M2" s="154"/>
-      <c r="N2" s="154"/>
-      <c r="O2" s="155"/>
-      <c r="P2" s="156" t="str">
+      <c r="L2" s="157"/>
+      <c r="M2" s="157"/>
+      <c r="N2" s="157"/>
+      <c r="O2" s="158"/>
+      <c r="P2" s="159" t="str">
         <f>Overview!P2</f>
         <v>SC Name</v>
       </c>
-      <c r="Q2" s="154"/>
-      <c r="R2" s="154"/>
-      <c r="S2" s="154"/>
-      <c r="T2" s="155"/>
-      <c r="U2" s="156" t="str">
+      <c r="Q2" s="157"/>
+      <c r="R2" s="157"/>
+      <c r="S2" s="157"/>
+      <c r="T2" s="158"/>
+      <c r="U2" s="159" t="str">
         <f>Overview!U2</f>
         <v>Template_DD_v1.0.xlsx</v>
       </c>
-      <c r="V2" s="154"/>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
-      <c r="Z2" s="154"/>
-      <c r="AA2" s="154"/>
-      <c r="AB2" s="154"/>
-      <c r="AC2" s="154"/>
-      <c r="AD2" s="155"/>
-      <c r="AE2" s="157">
+      <c r="V2" s="157"/>
+      <c r="W2" s="157"/>
+      <c r="X2" s="157"/>
+      <c r="Y2" s="157"/>
+      <c r="Z2" s="157"/>
+      <c r="AA2" s="157"/>
+      <c r="AB2" s="157"/>
+      <c r="AC2" s="157"/>
+      <c r="AD2" s="158"/>
+      <c r="AE2" s="151">
         <f>Overview!AI2</f>
         <v>45701</v>
       </c>
-      <c r="AF2" s="158"/>
-      <c r="AG2" s="158"/>
-      <c r="AH2" s="158"/>
-      <c r="AI2" s="159"/>
-      <c r="AJ2" s="151" t="str">
+      <c r="AF2" s="152"/>
+      <c r="AG2" s="152"/>
+      <c r="AH2" s="152"/>
+      <c r="AI2" s="153"/>
+      <c r="AJ2" s="154" t="str">
         <f>Overview!AN2</f>
         <v>BangNT</v>
       </c>
-      <c r="AK2" s="152"/>
-      <c r="AL2" s="152"/>
-      <c r="AM2" s="152"/>
-      <c r="AN2" s="157">
+      <c r="AK2" s="155"/>
+      <c r="AL2" s="155"/>
+      <c r="AM2" s="155"/>
+      <c r="AN2" s="151">
         <f>Overview!AS2</f>
         <v>45707</v>
       </c>
-      <c r="AO2" s="158"/>
-      <c r="AP2" s="158"/>
-      <c r="AQ2" s="158"/>
-      <c r="AR2" s="159"/>
-      <c r="AS2" s="120" t="str">
+      <c r="AO2" s="152"/>
+      <c r="AP2" s="152"/>
+      <c r="AQ2" s="152"/>
+      <c r="AR2" s="153"/>
+      <c r="AS2" s="117" t="str">
         <f>Overview!AX2</f>
         <v>BangNT</v>
       </c>
-      <c r="AT2" s="120"/>
-      <c r="AU2" s="120"/>
-      <c r="AV2" s="120"/>
-      <c r="AW2" s="120"/>
-      <c r="AX2" s="157">
+      <c r="AT2" s="117"/>
+      <c r="AU2" s="117"/>
+      <c r="AV2" s="117"/>
+      <c r="AW2" s="117"/>
+      <c r="AX2" s="151">
         <f>Overview!BC2</f>
         <v>45701</v>
       </c>
-      <c r="AY2" s="158"/>
-      <c r="AZ2" s="158"/>
-      <c r="BA2" s="158"/>
-      <c r="BB2" s="159"/>
-      <c r="BC2" s="176" t="str">
+      <c r="AY2" s="152"/>
+      <c r="AZ2" s="152"/>
+      <c r="BA2" s="152"/>
+      <c r="BB2" s="153"/>
+      <c r="BC2" s="170" t="str">
         <f>Overview!BH2</f>
         <v>BangNT</v>
       </c>
-      <c r="BD2" s="176"/>
-      <c r="BE2" s="176"/>
-      <c r="BF2" s="176"/>
-      <c r="BG2" s="176"/>
-      <c r="BH2" s="176"/>
-      <c r="BI2" s="176"/>
-      <c r="BJ2" s="176"/>
-      <c r="BK2" s="176"/>
-      <c r="BL2" s="176"/>
-      <c r="BM2" s="176"/>
-      <c r="BN2" s="176"/>
-      <c r="BO2" s="176"/>
-      <c r="BP2" s="176"/>
-      <c r="BQ2" s="176"/>
-      <c r="BR2" s="176"/>
-      <c r="BS2" s="176"/>
-      <c r="BT2" s="176"/>
+      <c r="BD2" s="170"/>
+      <c r="BE2" s="170"/>
+      <c r="BF2" s="170"/>
+      <c r="BG2" s="170"/>
+      <c r="BH2" s="170"/>
+      <c r="BI2" s="170"/>
+      <c r="BJ2" s="170"/>
+      <c r="BK2" s="170"/>
+      <c r="BL2" s="170"/>
+      <c r="BM2" s="170"/>
+      <c r="BN2" s="170"/>
+      <c r="BO2" s="170"/>
+      <c r="BP2" s="170"/>
+      <c r="BQ2" s="170"/>
+      <c r="BR2" s="170"/>
+      <c r="BS2" s="170"/>
+      <c r="BT2" s="170"/>
     </row>
     <row r="3" spans="1:72" s="4" customFormat="1" ht="10.5" customHeight="1">
       <c r="A3" s="2"/>
@@ -6018,10 +6589,10 @@
     </row>
     <row r="8" spans="1:72" s="57" customFormat="1" ht="12" customHeight="1">
       <c r="A8" s="56"/>
-      <c r="C8" s="166">
+      <c r="C8" s="160">
         <v>1</v>
       </c>
-      <c r="D8" s="167"/>
+      <c r="D8" s="161"/>
       <c r="E8" s="65" t="s">
         <v>93</v>
       </c>
@@ -6420,14 +6991,14 @@
       <c r="A16" s="56"/>
       <c r="C16" s="73"/>
       <c r="E16" s="76"/>
-      <c r="F16" s="168" t="s">
+      <c r="F16" s="162" t="s">
         <v>68</v>
       </c>
-      <c r="G16" s="169"/>
-      <c r="H16" s="169"/>
-      <c r="I16" s="169"/>
-      <c r="J16" s="169"/>
-      <c r="K16" s="170"/>
+      <c r="G16" s="163"/>
+      <c r="H16" s="163"/>
+      <c r="I16" s="163"/>
+      <c r="J16" s="163"/>
+      <c r="K16" s="164"/>
       <c r="L16" s="67" t="s">
         <v>89</v>
       </c>
@@ -6492,12 +7063,12 @@
       <c r="A17" s="56"/>
       <c r="C17" s="73"/>
       <c r="E17" s="76"/>
-      <c r="F17" s="171"/>
-      <c r="G17" s="172"/>
-      <c r="H17" s="172"/>
-      <c r="I17" s="172"/>
-      <c r="J17" s="172"/>
-      <c r="K17" s="173"/>
+      <c r="F17" s="165"/>
+      <c r="G17" s="166"/>
+      <c r="H17" s="166"/>
+      <c r="I17" s="166"/>
+      <c r="J17" s="166"/>
+      <c r="K17" s="167"/>
       <c r="L17" s="67" t="s">
         <v>90</v>
       </c>
@@ -7142,56 +7713,56 @@
       <c r="R31" s="66"/>
       <c r="S31" s="66"/>
       <c r="T31" s="68"/>
-      <c r="U31" s="160" t="s">
+      <c r="U31" s="171" t="s">
         <v>72</v>
       </c>
-      <c r="V31" s="161"/>
-      <c r="W31" s="161"/>
-      <c r="X31" s="161"/>
-      <c r="Y31" s="161"/>
-      <c r="Z31" s="161"/>
-      <c r="AA31" s="161"/>
-      <c r="AB31" s="161"/>
-      <c r="AC31" s="161"/>
-      <c r="AD31" s="161"/>
-      <c r="AE31" s="161"/>
-      <c r="AF31" s="162"/>
-      <c r="AG31" s="160" t="s">
+      <c r="V31" s="172"/>
+      <c r="W31" s="172"/>
+      <c r="X31" s="172"/>
+      <c r="Y31" s="172"/>
+      <c r="Z31" s="172"/>
+      <c r="AA31" s="172"/>
+      <c r="AB31" s="172"/>
+      <c r="AC31" s="172"/>
+      <c r="AD31" s="172"/>
+      <c r="AE31" s="172"/>
+      <c r="AF31" s="173"/>
+      <c r="AG31" s="171" t="s">
         <v>83</v>
       </c>
-      <c r="AH31" s="161"/>
-      <c r="AI31" s="161"/>
-      <c r="AJ31" s="161"/>
-      <c r="AK31" s="161"/>
-      <c r="AL31" s="161"/>
-      <c r="AM31" s="161"/>
-      <c r="AN31" s="161"/>
-      <c r="AO31" s="161"/>
-      <c r="AP31" s="161"/>
-      <c r="AQ31" s="161"/>
-      <c r="AR31" s="162"/>
-      <c r="AS31" s="163" t="s">
+      <c r="AH31" s="172"/>
+      <c r="AI31" s="172"/>
+      <c r="AJ31" s="172"/>
+      <c r="AK31" s="172"/>
+      <c r="AL31" s="172"/>
+      <c r="AM31" s="172"/>
+      <c r="AN31" s="172"/>
+      <c r="AO31" s="172"/>
+      <c r="AP31" s="172"/>
+      <c r="AQ31" s="172"/>
+      <c r="AR31" s="173"/>
+      <c r="AS31" s="174" t="s">
         <v>72</v>
       </c>
-      <c r="AT31" s="164"/>
-      <c r="AU31" s="164"/>
-      <c r="AV31" s="164"/>
-      <c r="AW31" s="164"/>
-      <c r="AX31" s="164"/>
-      <c r="AY31" s="164"/>
-      <c r="AZ31" s="164"/>
-      <c r="BA31" s="164"/>
-      <c r="BB31" s="164"/>
-      <c r="BC31" s="164"/>
-      <c r="BD31" s="164"/>
-      <c r="BE31" s="164"/>
-      <c r="BF31" s="164"/>
-      <c r="BG31" s="164"/>
-      <c r="BH31" s="164"/>
-      <c r="BI31" s="164"/>
-      <c r="BJ31" s="164"/>
-      <c r="BK31" s="164"/>
-      <c r="BL31" s="165"/>
+      <c r="AT31" s="175"/>
+      <c r="AU31" s="175"/>
+      <c r="AV31" s="175"/>
+      <c r="AW31" s="175"/>
+      <c r="AX31" s="175"/>
+      <c r="AY31" s="175"/>
+      <c r="AZ31" s="175"/>
+      <c r="BA31" s="175"/>
+      <c r="BB31" s="175"/>
+      <c r="BC31" s="175"/>
+      <c r="BD31" s="175"/>
+      <c r="BE31" s="175"/>
+      <c r="BF31" s="175"/>
+      <c r="BG31" s="175"/>
+      <c r="BH31" s="175"/>
+      <c r="BI31" s="175"/>
+      <c r="BJ31" s="175"/>
+      <c r="BK31" s="175"/>
+      <c r="BL31" s="176"/>
       <c r="BR31" s="84"/>
       <c r="BT31" s="64"/>
     </row>
@@ -7220,56 +7791,56 @@
       <c r="R32" s="66"/>
       <c r="S32" s="66"/>
       <c r="T32" s="68"/>
-      <c r="U32" s="160" t="s">
+      <c r="U32" s="171" t="s">
         <v>72</v>
       </c>
-      <c r="V32" s="161"/>
-      <c r="W32" s="161"/>
-      <c r="X32" s="161"/>
-      <c r="Y32" s="161"/>
-      <c r="Z32" s="161"/>
-      <c r="AA32" s="161"/>
-      <c r="AB32" s="161"/>
-      <c r="AC32" s="161"/>
-      <c r="AD32" s="161"/>
-      <c r="AE32" s="161"/>
-      <c r="AF32" s="162"/>
-      <c r="AG32" s="160" t="s">
+      <c r="V32" s="172"/>
+      <c r="W32" s="172"/>
+      <c r="X32" s="172"/>
+      <c r="Y32" s="172"/>
+      <c r="Z32" s="172"/>
+      <c r="AA32" s="172"/>
+      <c r="AB32" s="172"/>
+      <c r="AC32" s="172"/>
+      <c r="AD32" s="172"/>
+      <c r="AE32" s="172"/>
+      <c r="AF32" s="173"/>
+      <c r="AG32" s="171" t="s">
         <v>83</v>
       </c>
-      <c r="AH32" s="161"/>
-      <c r="AI32" s="161"/>
-      <c r="AJ32" s="161"/>
-      <c r="AK32" s="161"/>
-      <c r="AL32" s="161"/>
-      <c r="AM32" s="161"/>
-      <c r="AN32" s="161"/>
-      <c r="AO32" s="161"/>
-      <c r="AP32" s="161"/>
-      <c r="AQ32" s="161"/>
-      <c r="AR32" s="162"/>
-      <c r="AS32" s="163" t="s">
+      <c r="AH32" s="172"/>
+      <c r="AI32" s="172"/>
+      <c r="AJ32" s="172"/>
+      <c r="AK32" s="172"/>
+      <c r="AL32" s="172"/>
+      <c r="AM32" s="172"/>
+      <c r="AN32" s="172"/>
+      <c r="AO32" s="172"/>
+      <c r="AP32" s="172"/>
+      <c r="AQ32" s="172"/>
+      <c r="AR32" s="173"/>
+      <c r="AS32" s="174" t="s">
         <v>72</v>
       </c>
-      <c r="AT32" s="164"/>
-      <c r="AU32" s="164"/>
-      <c r="AV32" s="164"/>
-      <c r="AW32" s="164"/>
-      <c r="AX32" s="164"/>
-      <c r="AY32" s="164"/>
-      <c r="AZ32" s="164"/>
-      <c r="BA32" s="164"/>
-      <c r="BB32" s="164"/>
-      <c r="BC32" s="164"/>
-      <c r="BD32" s="164"/>
-      <c r="BE32" s="164"/>
-      <c r="BF32" s="164"/>
-      <c r="BG32" s="164"/>
-      <c r="BH32" s="164"/>
-      <c r="BI32" s="164"/>
-      <c r="BJ32" s="164"/>
-      <c r="BK32" s="164"/>
-      <c r="BL32" s="165"/>
+      <c r="AT32" s="175"/>
+      <c r="AU32" s="175"/>
+      <c r="AV32" s="175"/>
+      <c r="AW32" s="175"/>
+      <c r="AX32" s="175"/>
+      <c r="AY32" s="175"/>
+      <c r="AZ32" s="175"/>
+      <c r="BA32" s="175"/>
+      <c r="BB32" s="175"/>
+      <c r="BC32" s="175"/>
+      <c r="BD32" s="175"/>
+      <c r="BE32" s="175"/>
+      <c r="BF32" s="175"/>
+      <c r="BG32" s="175"/>
+      <c r="BH32" s="175"/>
+      <c r="BI32" s="175"/>
+      <c r="BJ32" s="175"/>
+      <c r="BK32" s="175"/>
+      <c r="BL32" s="176"/>
       <c r="BR32" s="84"/>
       <c r="BT32" s="64"/>
     </row>
@@ -7436,10 +8007,10 @@
     </row>
     <row r="37" spans="1:72" s="57" customFormat="1" ht="12" customHeight="1">
       <c r="A37" s="56"/>
-      <c r="C37" s="166">
+      <c r="C37" s="160">
         <v>1</v>
       </c>
-      <c r="D37" s="167"/>
+      <c r="D37" s="161"/>
       <c r="E37" s="65" t="s">
         <v>96</v>
       </c>
@@ -7838,14 +8409,14 @@
       <c r="A45" s="56"/>
       <c r="C45" s="73"/>
       <c r="E45" s="76"/>
-      <c r="F45" s="168" t="s">
+      <c r="F45" s="162" t="s">
         <v>68</v>
       </c>
-      <c r="G45" s="169"/>
-      <c r="H45" s="169"/>
-      <c r="I45" s="169"/>
-      <c r="J45" s="169"/>
-      <c r="K45" s="170"/>
+      <c r="G45" s="163"/>
+      <c r="H45" s="163"/>
+      <c r="I45" s="163"/>
+      <c r="J45" s="163"/>
+      <c r="K45" s="164"/>
       <c r="L45" s="67" t="s">
         <v>89</v>
       </c>
@@ -7910,12 +8481,12 @@
       <c r="A46" s="56"/>
       <c r="C46" s="73"/>
       <c r="E46" s="76"/>
-      <c r="F46" s="171"/>
-      <c r="G46" s="172"/>
-      <c r="H46" s="172"/>
-      <c r="I46" s="172"/>
-      <c r="J46" s="172"/>
-      <c r="K46" s="173"/>
+      <c r="F46" s="165"/>
+      <c r="G46" s="166"/>
+      <c r="H46" s="166"/>
+      <c r="I46" s="166"/>
+      <c r="J46" s="166"/>
+      <c r="K46" s="167"/>
       <c r="L46" s="67" t="s">
         <v>90</v>
       </c>
@@ -8560,56 +9131,56 @@
       <c r="R60" s="66"/>
       <c r="S60" s="66"/>
       <c r="T60" s="68"/>
-      <c r="U60" s="160" t="s">
+      <c r="U60" s="171" t="s">
         <v>72</v>
       </c>
-      <c r="V60" s="161"/>
-      <c r="W60" s="161"/>
-      <c r="X60" s="161"/>
-      <c r="Y60" s="161"/>
-      <c r="Z60" s="161"/>
-      <c r="AA60" s="161"/>
-      <c r="AB60" s="161"/>
-      <c r="AC60" s="161"/>
-      <c r="AD60" s="161"/>
-      <c r="AE60" s="161"/>
-      <c r="AF60" s="162"/>
-      <c r="AG60" s="160" t="s">
+      <c r="V60" s="172"/>
+      <c r="W60" s="172"/>
+      <c r="X60" s="172"/>
+      <c r="Y60" s="172"/>
+      <c r="Z60" s="172"/>
+      <c r="AA60" s="172"/>
+      <c r="AB60" s="172"/>
+      <c r="AC60" s="172"/>
+      <c r="AD60" s="172"/>
+      <c r="AE60" s="172"/>
+      <c r="AF60" s="173"/>
+      <c r="AG60" s="171" t="s">
         <v>83</v>
       </c>
-      <c r="AH60" s="161"/>
-      <c r="AI60" s="161"/>
-      <c r="AJ60" s="161"/>
-      <c r="AK60" s="161"/>
-      <c r="AL60" s="161"/>
-      <c r="AM60" s="161"/>
-      <c r="AN60" s="161"/>
-      <c r="AO60" s="161"/>
-      <c r="AP60" s="161"/>
-      <c r="AQ60" s="161"/>
-      <c r="AR60" s="162"/>
-      <c r="AS60" s="163" t="s">
+      <c r="AH60" s="172"/>
+      <c r="AI60" s="172"/>
+      <c r="AJ60" s="172"/>
+      <c r="AK60" s="172"/>
+      <c r="AL60" s="172"/>
+      <c r="AM60" s="172"/>
+      <c r="AN60" s="172"/>
+      <c r="AO60" s="172"/>
+      <c r="AP60" s="172"/>
+      <c r="AQ60" s="172"/>
+      <c r="AR60" s="173"/>
+      <c r="AS60" s="174" t="s">
         <v>72</v>
       </c>
-      <c r="AT60" s="164"/>
-      <c r="AU60" s="164"/>
-      <c r="AV60" s="164"/>
-      <c r="AW60" s="164"/>
-      <c r="AX60" s="164"/>
-      <c r="AY60" s="164"/>
-      <c r="AZ60" s="164"/>
-      <c r="BA60" s="164"/>
-      <c r="BB60" s="164"/>
-      <c r="BC60" s="164"/>
-      <c r="BD60" s="164"/>
-      <c r="BE60" s="164"/>
-      <c r="BF60" s="164"/>
-      <c r="BG60" s="164"/>
-      <c r="BH60" s="164"/>
-      <c r="BI60" s="164"/>
-      <c r="BJ60" s="164"/>
-      <c r="BK60" s="164"/>
-      <c r="BL60" s="165"/>
+      <c r="AT60" s="175"/>
+      <c r="AU60" s="175"/>
+      <c r="AV60" s="175"/>
+      <c r="AW60" s="175"/>
+      <c r="AX60" s="175"/>
+      <c r="AY60" s="175"/>
+      <c r="AZ60" s="175"/>
+      <c r="BA60" s="175"/>
+      <c r="BB60" s="175"/>
+      <c r="BC60" s="175"/>
+      <c r="BD60" s="175"/>
+      <c r="BE60" s="175"/>
+      <c r="BF60" s="175"/>
+      <c r="BG60" s="175"/>
+      <c r="BH60" s="175"/>
+      <c r="BI60" s="175"/>
+      <c r="BJ60" s="175"/>
+      <c r="BK60" s="175"/>
+      <c r="BL60" s="176"/>
       <c r="BR60" s="84"/>
       <c r="BT60" s="64"/>
     </row>
@@ -8638,56 +9209,56 @@
       <c r="R61" s="66"/>
       <c r="S61" s="66"/>
       <c r="T61" s="68"/>
-      <c r="U61" s="160" t="s">
+      <c r="U61" s="171" t="s">
         <v>72</v>
       </c>
-      <c r="V61" s="161"/>
-      <c r="W61" s="161"/>
-      <c r="X61" s="161"/>
-      <c r="Y61" s="161"/>
-      <c r="Z61" s="161"/>
-      <c r="AA61" s="161"/>
-      <c r="AB61" s="161"/>
-      <c r="AC61" s="161"/>
-      <c r="AD61" s="161"/>
-      <c r="AE61" s="161"/>
-      <c r="AF61" s="162"/>
-      <c r="AG61" s="160" t="s">
+      <c r="V61" s="172"/>
+      <c r="W61" s="172"/>
+      <c r="X61" s="172"/>
+      <c r="Y61" s="172"/>
+      <c r="Z61" s="172"/>
+      <c r="AA61" s="172"/>
+      <c r="AB61" s="172"/>
+      <c r="AC61" s="172"/>
+      <c r="AD61" s="172"/>
+      <c r="AE61" s="172"/>
+      <c r="AF61" s="173"/>
+      <c r="AG61" s="171" t="s">
         <v>83</v>
       </c>
-      <c r="AH61" s="161"/>
-      <c r="AI61" s="161"/>
-      <c r="AJ61" s="161"/>
-      <c r="AK61" s="161"/>
-      <c r="AL61" s="161"/>
-      <c r="AM61" s="161"/>
-      <c r="AN61" s="161"/>
-      <c r="AO61" s="161"/>
-      <c r="AP61" s="161"/>
-      <c r="AQ61" s="161"/>
-      <c r="AR61" s="162"/>
-      <c r="AS61" s="163" t="s">
+      <c r="AH61" s="172"/>
+      <c r="AI61" s="172"/>
+      <c r="AJ61" s="172"/>
+      <c r="AK61" s="172"/>
+      <c r="AL61" s="172"/>
+      <c r="AM61" s="172"/>
+      <c r="AN61" s="172"/>
+      <c r="AO61" s="172"/>
+      <c r="AP61" s="172"/>
+      <c r="AQ61" s="172"/>
+      <c r="AR61" s="173"/>
+      <c r="AS61" s="174" t="s">
         <v>72</v>
       </c>
-      <c r="AT61" s="164"/>
-      <c r="AU61" s="164"/>
-      <c r="AV61" s="164"/>
-      <c r="AW61" s="164"/>
-      <c r="AX61" s="164"/>
-      <c r="AY61" s="164"/>
-      <c r="AZ61" s="164"/>
-      <c r="BA61" s="164"/>
-      <c r="BB61" s="164"/>
-      <c r="BC61" s="164"/>
-      <c r="BD61" s="164"/>
-      <c r="BE61" s="164"/>
-      <c r="BF61" s="164"/>
-      <c r="BG61" s="164"/>
-      <c r="BH61" s="164"/>
-      <c r="BI61" s="164"/>
-      <c r="BJ61" s="164"/>
-      <c r="BK61" s="164"/>
-      <c r="BL61" s="165"/>
+      <c r="AT61" s="175"/>
+      <c r="AU61" s="175"/>
+      <c r="AV61" s="175"/>
+      <c r="AW61" s="175"/>
+      <c r="AX61" s="175"/>
+      <c r="AY61" s="175"/>
+      <c r="AZ61" s="175"/>
+      <c r="BA61" s="175"/>
+      <c r="BB61" s="175"/>
+      <c r="BC61" s="175"/>
+      <c r="BD61" s="175"/>
+      <c r="BE61" s="175"/>
+      <c r="BF61" s="175"/>
+      <c r="BG61" s="175"/>
+      <c r="BH61" s="175"/>
+      <c r="BI61" s="175"/>
+      <c r="BJ61" s="175"/>
+      <c r="BK61" s="175"/>
+      <c r="BL61" s="176"/>
       <c r="BR61" s="84"/>
       <c r="BT61" s="64"/>
     </row>
@@ -8766,20 +9337,14 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="F16:K17"/>
-    <mergeCell ref="AE1:AI1"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="K1:O1"/>
-    <mergeCell ref="P1:T1"/>
-    <mergeCell ref="U1:AD1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="K2:O2"/>
-    <mergeCell ref="P2:T2"/>
-    <mergeCell ref="U2:AD2"/>
-    <mergeCell ref="AE2:AI2"/>
+    <mergeCell ref="U61:AF61"/>
+    <mergeCell ref="AG61:AR61"/>
+    <mergeCell ref="AS61:BL61"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="F45:K46"/>
+    <mergeCell ref="U60:AF60"/>
+    <mergeCell ref="AG60:AR60"/>
+    <mergeCell ref="AS60:BL60"/>
     <mergeCell ref="BC1:BT1"/>
     <mergeCell ref="BC2:BT2"/>
     <mergeCell ref="U32:AF32"/>
@@ -8796,14 +9361,20 @@
     <mergeCell ref="AN2:AR2"/>
     <mergeCell ref="AS2:AW2"/>
     <mergeCell ref="AX2:BB2"/>
-    <mergeCell ref="U61:AF61"/>
-    <mergeCell ref="AG61:AR61"/>
-    <mergeCell ref="AS61:BL61"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="F45:K46"/>
-    <mergeCell ref="U60:AF60"/>
-    <mergeCell ref="AG60:AR60"/>
-    <mergeCell ref="AS60:BL60"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="F16:K17"/>
+    <mergeCell ref="AE1:AI1"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="P1:T1"/>
+    <mergeCell ref="U1:AD1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="K2:O2"/>
+    <mergeCell ref="P2:T2"/>
+    <mergeCell ref="U2:AD2"/>
+    <mergeCell ref="AE2:AI2"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="77" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -8813,7 +9384,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="B2:B12"/>
   <sheetFormatPr defaultRowHeight="13.2"/>

</xml_diff>